<commit_message>
Update new animation + fx
</commit_message>
<xml_diff>
--- a/LocalizationStringTable.xlsx
+++ b/LocalizationStringTable.xlsx
@@ -711,11 +711,11 @@
         <v>Control UI_Bet Area</v>
       </c>
       <c r="C9" t="str" xml:space="preserve">
-        <v xml:space="preserve">CLICK TO CHANGE BETWEEN_x000d_
+        <v xml:space="preserve">CLICK TO CHANGE BETWEEN
 MONEY AND COIN VIEW</v>
       </c>
       <c r="D9" t="str" xml:space="preserve">
-        <v xml:space="preserve">클릭하면 머니 보기와 코인 보기_x000d_
+        <v xml:space="preserve">클릭하면 머니 보기와 코인 보기
 상태가 전환됩니다.</v>
       </c>
       <c r="E9" t="str">
@@ -734,15 +734,15 @@
         <v>คลิกเพื่อสลับระหว่างมุมมองเงินและเหรียญ</v>
       </c>
       <c r="J9" t="str" xml:space="preserve">
-        <v xml:space="preserve">CLICK TO CHANGE BETWEEN_x000d_
+        <v xml:space="preserve">CLICK TO CHANGE BETWEEN
 MONEY AND COIN VIEW</v>
       </c>
       <c r="K9" t="str" xml:space="preserve">
-        <v xml:space="preserve">KLIK UNTUK BERTUKAR ANTARA_x000d_
+        <v xml:space="preserve">KLIK UNTUK BERTUKAR ANTARA
 PAPARAN WANG DAN KOIN</v>
       </c>
       <c r="L9" t="str" xml:space="preserve">
-        <v xml:space="preserve">NHẤP ĐỂ CHUYỂN GIỮA_x000d_
+        <v xml:space="preserve">NHẤP ĐỂ CHUYỂN GIỮA
 CHẾ ĐỘ XEM TIỀN VÀ XU</v>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
         <v>System Setting Pop-up</v>
       </c>
       <c r="C30" t="str" xml:space="preserve">
-        <v xml:space="preserve">TURN ON OR OFF _x000d_
+        <v xml:space="preserve">TURN ON OR OFF 
 THE GAME MUSIC</v>
       </c>
       <c r="D30" t="str">
@@ -1536,15 +1536,15 @@
         <v>เปิดหรือปิดเพลงของเกม</v>
       </c>
       <c r="J30" t="str" xml:space="preserve">
-        <v xml:space="preserve">TURN ON OR OFF _x000d_
+        <v xml:space="preserve">TURN ON OR OFF 
 THE GAME MUSIC</v>
       </c>
       <c r="K30" t="str" xml:space="preserve">
-        <v xml:space="preserve">HIDUPKAN ATAU MATIKAN_x000d_
+        <v xml:space="preserve">HIDUPKAN ATAU MATIKAN
 MUZIK PERMAINAN</v>
       </c>
       <c r="L30" t="str" xml:space="preserve">
-        <v xml:space="preserve">BẬT HOẶC TẮT_x000d_
+        <v xml:space="preserve">BẬT HOẶC TẮT
 NHẠC CỦA TRÒ CHƠI</v>
       </c>
     </row>
@@ -1594,7 +1594,7 @@
         <v>System Setting Pop-up</v>
       </c>
       <c r="C32" t="str" xml:space="preserve">
-        <v xml:space="preserve">TURN ON OR OFF_x000d_
+        <v xml:space="preserve">TURN ON OR OFF
 GAME WIN BROAD CASTING</v>
       </c>
       <c r="D32" t="str">
@@ -1616,15 +1616,15 @@
         <v>เปิด / ปิด การประกาศชัยชนะในเกม</v>
       </c>
       <c r="J32" t="str" xml:space="preserve">
-        <v xml:space="preserve">TURN ON OR OFF_x000d_
+        <v xml:space="preserve">TURN ON OR OFF
 GAME WIN BROAD CASTING</v>
       </c>
       <c r="K32" t="str" xml:space="preserve">
-        <v xml:space="preserve">HIDUPKAN ATAU MATIKAN_x000d_
+        <v xml:space="preserve">HIDUPKAN ATAU MATIKAN
 SIARAN KEMENANGAN PERMAINAN</v>
       </c>
       <c r="L32" t="str" xml:space="preserve">
-        <v xml:space="preserve">BẬT HOẶC TẮT_x000d_
+        <v xml:space="preserve">BẬT HOẶC TẮT
 PHÁT SÓNG CHIẾN THẮNG TRONG TRÒ CHƠI</v>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
         <v>System Setting Pop-up</v>
       </c>
       <c r="C34" t="str" xml:space="preserve">
-        <v xml:space="preserve">SHOW THE INTRO SCREEN BEFORE _x000d_
+        <v xml:space="preserve">SHOW THE INTRO SCREEN BEFORE 
 STARTING THE GAME</v>
       </c>
       <c r="D34" t="str">
@@ -1696,15 +1696,15 @@
         <v>แสดงหน้าจอแนะนำก่อนเริ่มเกม</v>
       </c>
       <c r="J34" t="str" xml:space="preserve">
-        <v xml:space="preserve">SHOW THE INTRO SCREEN BEFORE _x000d_
+        <v xml:space="preserve">SHOW THE INTRO SCREEN BEFORE 
 STARTING THE GAME</v>
       </c>
       <c r="K34" t="str" xml:space="preserve">
-        <v xml:space="preserve">TUNJUKKAN SKRIN INTRO SEBELUM_x000d_
+        <v xml:space="preserve">TUNJUKKAN SKRIN INTRO SEBELUM
 MEMULAKAN PERMAINAN</v>
       </c>
       <c r="L34" t="str" xml:space="preserve">
-        <v xml:space="preserve">HIỂN THỊ MÀN HÌNH GIỚI THIỆU TRƯỚC_x000d_
+        <v xml:space="preserve">HIỂN THỊ MÀN HÌNH GIỚI THIỆU TRƯỚC
 KHI BẮT ĐẦU TRÒ CHƠI</v>
       </c>
     </row>
@@ -1754,7 +1754,7 @@
         <v>System Setting Pop-up</v>
       </c>
       <c r="C36" t="str" xml:space="preserve">
-        <v xml:space="preserve">TURN ON OR OFF _x000d_
+        <v xml:space="preserve">TURN ON OR OFF 
 THE GAME SOUND</v>
       </c>
       <c r="D36" t="str">
@@ -1776,15 +1776,15 @@
         <v>เปิดหรือปิดเสียงของเกม</v>
       </c>
       <c r="J36" t="str" xml:space="preserve">
-        <v xml:space="preserve">TURN ON OR OFF _x000d_
+        <v xml:space="preserve">TURN ON OR OFF 
 THE GAME SOUND</v>
       </c>
       <c r="K36" t="str" xml:space="preserve">
-        <v xml:space="preserve">HIDUPKAN ATAU MATIKAN_x000d_
+        <v xml:space="preserve">HIDUPKAN ATAU MATIKAN
 BUNYI PERMAINAN</v>
       </c>
       <c r="L36" t="str" xml:space="preserve">
-        <v xml:space="preserve">BẬT HOẶC TẮT_x000d_
+        <v xml:space="preserve">BẬT HOẶC TẮT
 ÂM THANH CỦA TRÒ CHƠI</v>
       </c>
     </row>
@@ -2138,51 +2138,51 @@
         <v>System Message Pop-up</v>
       </c>
       <c r="C46" t="str" xml:space="preserve">
-        <v xml:space="preserve">Please recharge funds in your cash wallet._x000d_
-If the balance is not updated after recharging,_x000d_
+        <v xml:space="preserve">Please recharge funds in your cash wallet.
+If the balance is not updated after recharging,
 please refresh your cash wallet.</v>
       </c>
       <c r="D46" t="str" xml:space="preserve">
-        <v xml:space="preserve">캐시 지갑에 금액을 층전해주세요._x000d_
-충전 후에도 잔액이 업데이트 되지 않으면_x000d_
+        <v xml:space="preserve">캐시 지갑에 금액을 층전해주세요.
+충전 후에도 잔액이 업데이트 되지 않으면
 캐시 지갑을 새로고침해 주세요.</v>
       </c>
       <c r="E46" t="str" xml:space="preserve">
-        <v xml:space="preserve">请为您的现金钱包充值。_x000d_
-如果充值后余额未更新，_x000d_
+        <v xml:space="preserve">请为您的现金钱包充值。
+如果充值后余额未更新，
 请刷新您的现金钱包。</v>
       </c>
       <c r="F46" t="str" xml:space="preserve">
-        <v xml:space="preserve">請為您的現金錢包充值。_x000d_
-若充值後餘額未更新，_x000d_
+        <v xml:space="preserve">請為您的現金錢包充值。
+若充值後餘額未更新，
 請重新整理您的現金錢包。</v>
       </c>
       <c r="G46" t="str" xml:space="preserve">
-        <v xml:space="preserve">Pakilagyan ng pondo ang iyong cash wallet. _x000d_
-Kung hindi pa rin nag-a-update ang balanse pagkatapos mag-recharge, _x000d_
+        <v xml:space="preserve">Pakilagyan ng pondo ang iyong cash wallet. 
+Kung hindi pa rin nag-a-update ang balanse pagkatapos mag-recharge, 
 paki-refresh ang iyong cash wallet.</v>
       </c>
       <c r="H46" t="str" xml:space="preserve">
-        <v xml:space="preserve">キャッシュウォレットにチャージしてください。_x000d_
-チャージ後も残高が更新されない場合は、_x000d_
+        <v xml:space="preserve">キャッシュウォレットにチャージしてください。
+チャージ後も残高が更新されない場合は、
 キャッシュウォレットを更新してください。</v>
       </c>
       <c r="I46" t="str">
         <v>กรุณาเติมเงินเข้ากระเป๋าเงินสดของคุณ หากยอดคงเหลือไม่อัปเดตหลังจากเติมเงิน กรุณารีเฟรชกระเป๋าเงินสดของคุณ</v>
       </c>
       <c r="J46" t="str" xml:space="preserve">
-        <v xml:space="preserve">Please recharge funds in your cash wallet._x000d_
-If the balance is not updated after recharging,_x000d_
+        <v xml:space="preserve">Please recharge funds in your cash wallet.
+If the balance is not updated after recharging,
 please refresh your cash wallet.</v>
       </c>
       <c r="K46" t="str" xml:space="preserve">
-        <v xml:space="preserve">Sila tambah dana ke dalam cash wallet anda._x000d_
-Jika baki tidak dikemas kini selepas tambah nilai,_x000d_
+        <v xml:space="preserve">Sila tambah dana ke dalam cash wallet anda.
+Jika baki tidak dikemas kini selepas tambah nilai,
 sila muat semula cash wallet anda.</v>
       </c>
       <c r="L46" t="str" xml:space="preserve">
-        <v xml:space="preserve">Vui lòng nạp tiền vào ví tiền mặt của bạn._x000d_
-Nếu số dư không được cập nhật sau khi nạp,_x000d_
+        <v xml:space="preserve">Vui lòng nạp tiền vào ví tiền mặt của bạn.
+Nếu số dư không được cập nhật sau khi nạp,
 vui lòng làm mới ví tiền mặt của bạn.</v>
       </c>
     </row>
@@ -2232,42 +2232,42 @@
         <v>System Message Pop-up</v>
       </c>
       <c r="C48" t="str" xml:space="preserve">
-        <v xml:space="preserve">Wrong Parsheet Symbol ID._x000d_
+        <v xml:space="preserve">Wrong Parsheet Symbol ID.
 You have been disconnected from the server.</v>
       </c>
       <c r="D48" t="str" xml:space="preserve">
-        <v xml:space="preserve">잘못된 심볼 ID입니다._x000d_
+        <v xml:space="preserve">잘못된 심볼 ID입니다.
 서버와의 연결이 끊어졌습니다.</v>
       </c>
       <c r="E48" t="str" xml:space="preserve">
-        <v xml:space="preserve">Symbol ID错误。_x000d_
+        <v xml:space="preserve">Symbol ID错误。
 您已与服务器断开连接。</v>
       </c>
       <c r="F48" t="str" xml:space="preserve">
-        <v xml:space="preserve">Symbol ID 錯誤。_x000d_
+        <v xml:space="preserve">Symbol ID 錯誤。
 您已與伺服器中斷連線。</v>
       </c>
       <c r="G48" t="str" xml:space="preserve">
-        <v xml:space="preserve">Maling Symbol ID. _x000d_
+        <v xml:space="preserve">Maling Symbol ID. 
 Nadiskonekta ka mula sa server.</v>
       </c>
       <c r="H48" t="str" xml:space="preserve">
-        <v xml:space="preserve">Symbol ID が正しくありません。_x000d_
+        <v xml:space="preserve">Symbol ID が正しくありません。
 サーバーから切断されました。</v>
       </c>
       <c r="I48" t="str">
         <v>Symbol ID ไม่ถูกต้อง คุณถูกตัดการเชื่อมต่อจากเซิร์ฟเวอร์</v>
       </c>
       <c r="J48" t="str" xml:space="preserve">
-        <v xml:space="preserve">Wrong Parsheet Symbol ID._x000d_
+        <v xml:space="preserve">Wrong Parsheet Symbol ID.
 You have been disconnected from the server.</v>
       </c>
       <c r="K48" t="str" xml:space="preserve">
-        <v xml:space="preserve">Symbol ID tidak sah._x000d_
+        <v xml:space="preserve">Symbol ID tidak sah.
 Sambungan anda dengan pelayan telah terputus.</v>
       </c>
       <c r="L48" t="str" xml:space="preserve">
-        <v xml:space="preserve">Symbol ID không hợp lệ._x000d_
+        <v xml:space="preserve">Symbol ID không hợp lệ.
 Bạn đã bị ngắt kết nối khỏi máy chủ.</v>
       </c>
     </row>
@@ -2393,53 +2393,53 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C52" t="str" xml:space="preserve">
-        <v xml:space="preserve">Symbols pay left to right on adjacent reels._x000d_
-243 ways to win on every spin._x000d_
+        <v xml:space="preserve">Symbols pay left to right on adjacent reels.
+243 ways to win on every spin.
 Only the highest-paying combination per way is paid.</v>
       </c>
       <c r="D52" t="str" xml:space="preserve">
-        <v xml:space="preserve">심볼은 연속된 릴에서 좌측부터 우측으로 연결될 때 당첨 됩니다._x000d_
-매 스핀 마다 243 ways의 당첨 기회를 제공합니다._x000d_
+        <v xml:space="preserve">심볼은 연속된 릴에서 좌측부터 우측으로 연결될 때 당첨 됩니다.
+매 스핀 마다 243 ways의 당첨 기회를 제공합니다.
 동일한 ways에서는 가장 높은 당첨금만 지급 됩니다.</v>
       </c>
       <c r="E52" t="str" xml:space="preserve">
-        <v xml:space="preserve">符号需在相邻转轴上从左至右连续出现方可获胜。_x000d_
-每次旋转提供243种获胜方式。_x000d_
+        <v xml:space="preserve">符号需在相邻转轴上从左至右连续出现方可获胜。
+每次旋转提供243种获胜方式。
 每种获胜方式仅支付最高奖金组合。</v>
       </c>
       <c r="F52" t="str" xml:space="preserve">
-        <v xml:space="preserve">符號在相鄰轉軸上由左至右連續排列即可獲得派彩。_x000d_
-每次旋轉皆有243種獲勝方式。_x000d_
+        <v xml:space="preserve">符號在相鄰轉軸上由左至右連續排列即可獲得派彩。
+每次旋轉皆有243種獲勝方式。
 每種獲勝方式僅支付最高獎勵組合。</v>
       </c>
       <c r="G52" t="str" xml:space="preserve">
-        <v xml:space="preserve">Ang mga simbolo ay magbabayad mula kaliwa pakanan sa magkatabing reels._x000d_
-May 243 paraan upang manalo sa bawat spin._x000d_
+        <v xml:space="preserve">Ang mga simbolo ay magbabayad mula kaliwa pakanan sa magkatabing reels.
+May 243 paraan upang manalo sa bawat spin.
 Tanging ang pinakamataas na kombinasyong panalo sa bawat paraan ang babayaran.</v>
       </c>
       <c r="H52" t="str" xml:space="preserve">
-        <v xml:space="preserve">シンボルは隣接するリール上で左から右に揃うと配当が支払われます。_x000d_
-毎スピン243通りの勝利チャンスがあります。_x000d_
+        <v xml:space="preserve">シンボルは隣接するリール上で左から右に揃うと配当が支払われます。
+毎スピン243通りの勝利チャンスがあります。
 各配当ラインでは、最も高い配当の組み合わせのみが支払われます。</v>
       </c>
       <c r="I52" t="str" xml:space="preserve">
-        <v xml:space="preserve">สัญลักษณ์จะจ่ายรางวัลเมื่อเรียงต่อกันจากซ้ายไปขวาบนวงล้อที่อยู่ติดกัน_x000d_
-ทุกการหมุนมีโอกาสชนะได้ถึง 243 วิธี_x000d_
+        <v xml:space="preserve">สัญลักษณ์จะจ่ายรางวัลเมื่อเรียงต่อกันจากซ้ายไปขวาบนวงล้อที่อยู่ติดกัน
+ทุกการหมุนมีโอกาสชนะได้ถึง 243 วิธี
 แต่ละวิธีการชนะจะจ่ายเฉพาะชุดสัญลักษณ์ที่มีมูลค่าสูงสุดเท่านั้น</v>
       </c>
       <c r="J52" t="str" xml:space="preserve">
-        <v xml:space="preserve">Symbols pay left to right on adjacent reels._x000d_
-243 ways to win on every spin._x000d_
+        <v xml:space="preserve">Symbols pay left to right on adjacent reels.
+243 ways to win on every spin.
 Only the highest-paying combination per way is paid.</v>
       </c>
       <c r="K52" t="str" xml:space="preserve">
-        <v xml:space="preserve">Simbol membayar dari kiri ke kanan pada reel yang bersebelahan._x000d_
-243 cara untuk menang pada setiap spin._x000d_
+        <v xml:space="preserve">Simbol membayar dari kiri ke kanan pada reel yang bersebelahan.
+243 cara untuk menang pada setiap spin.
 Hanya kombinasi bayaran tertinggi bagi setiap cara akan dibayar.</v>
       </c>
       <c r="L52" t="str" xml:space="preserve">
-        <v xml:space="preserve">Các biểu tượng trả thưởng từ trái sang phải trên các reel liền kề._x000d_
-243 cách thắng ở mọi lượt quay._x000d_
+        <v xml:space="preserve">Các biểu tượng trả thưởng từ trái sang phải trên các reel liền kề.
+243 cách thắng ở mọi lượt quay.
 Chỉ tổ hợp trả thưởng cao nhất của mỗi cách thắng được chi trả.</v>
       </c>
     </row>
@@ -2489,43 +2489,43 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C54" t="str" xml:space="preserve">
-        <v xml:space="preserve">The Sakura Symbol acts as a Wild and substitutes for all symbols except Trail Symbols._x000d_
+        <v xml:space="preserve">The Sakura Symbol acts as a Wild and substitutes for all symbols except Trail Symbols.
 The Sakura Symbol appears on reels 2, 3, and 4 during the Base Game.</v>
       </c>
       <c r="D54" t="str" xml:space="preserve">
-        <v xml:space="preserve">사쿠라 심볼은 와일드 심볼로 동작하며, Trail Symbol을 제외한 모든 심볼을 대체합니다._x000d_
+        <v xml:space="preserve">사쿠라 심볼은 와일드 심볼로 동작하며, Trail Symbol을 제외한 모든 심볼을 대체합니다.
 사쿠라 심볼은 Base Game에서 2번, 3번, 4번 릴에 등장합니다.</v>
       </c>
       <c r="E54" t="str" xml:space="preserve">
-        <v xml:space="preserve">樱花符号可作为WILD使用，并可替代除Trail Symbol之外的所有符号。_x000d_
+        <v xml:space="preserve">樱花符号可作为WILD使用，并可替代除Trail Symbol之外的所有符号。
 樱花符号仅会在基础游戏（Base Game）的第2、3、4转轴上出现。</v>
       </c>
       <c r="F54" t="str" xml:space="preserve">
-        <v xml:space="preserve">櫻花符號可作為WILD使用，並可替代除Trail Symbol之外的所有符號。_x000d_
+        <v xml:space="preserve">櫻花符號可作為WILD使用，並可替代除Trail Symbol之外的所有符號。
 櫻花符號僅會在基本遊戲（Base Game）的第2、3、4轉軸上出現。</v>
       </c>
       <c r="G54" t="str" xml:space="preserve">
-        <v xml:space="preserve">Ang Sakura Symbol ay nagsisilbing Wild at maaaring pumalit sa lahat ng simbolo maliban sa mga Trail Symbol._x000d_
+        <v xml:space="preserve">Ang Sakura Symbol ay nagsisilbing Wild at maaaring pumalit sa lahat ng simbolo maliban sa mga Trail Symbol.
 Lumalabas ang Sakura Symbol sa reels 2, 3, at 4 sa panahon ng Base Game.</v>
       </c>
       <c r="H54" t="str" xml:space="preserve">
-        <v xml:space="preserve">サクラシンボルはWILDとして機能し、Trail Symbolを除くすべてのシンボルの代わりになります。_x000d_
+        <v xml:space="preserve">サクラシンボルはWILDとして機能し、Trail Symbolを除くすべてのシンボルの代わりになります。
 サクラシンボルはベースゲーム中のリール2、3、4に出現します。</v>
       </c>
       <c r="I54" t="str" xml:space="preserve">
-        <v xml:space="preserve">สัญลักษณ์ Sakura ทำหน้าที่เป็น Wild และสามารถแทนที่สัญลักษณ์ทั้งหมดได้ ยกเว้น Trail Symbol_x000d_
+        <v xml:space="preserve">สัญลักษณ์ Sakura ทำหน้าที่เป็น Wild และสามารถแทนที่สัญลักษณ์ทั้งหมดได้ ยกเว้น Trail Symbol
 สัญลักษณ์ Sakura จะปรากฏบนวงล้อที่ 2, 3 และ 4 ในระหว่าง Base Game</v>
       </c>
       <c r="J54" t="str" xml:space="preserve">
-        <v xml:space="preserve">The Sakura Symbol acts as a Wild and substitutes for all symbols except Trail Symbols._x000d_
+        <v xml:space="preserve">The Sakura Symbol acts as a Wild and substitutes for all symbols except Trail Symbols.
 The Sakura Symbol appears on reels 2, 3, and 4 during the Base Game.</v>
       </c>
       <c r="K54" t="str" xml:space="preserve">
-        <v xml:space="preserve">Sakura Symbol bertindak sebagai Wild dan menggantikan semua simbol kecuali Trail Symbol._x000d_
+        <v xml:space="preserve">Sakura Symbol bertindak sebagai Wild dan menggantikan semua simbol kecuali Trail Symbol.
 Sakura Symbol muncul pada reel 2, 3 dan 4 semasa Base Game.</v>
       </c>
       <c r="L54" t="str" xml:space="preserve">
-        <v xml:space="preserve">Sakura Symbol hoạt động như Wild và thay thế cho tất cả các biểu tượng, ngoại trừ Trail Symbol._x000d_
+        <v xml:space="preserve">Sakura Symbol hoạt động như Wild và thay thế cho tất cả các biểu tượng, ngoại trừ Trail Symbol.
 Sakura Symbol xuất hiện trên reel 2, 3 và 4 trong Base Game.</v>
       </c>
     </row>
@@ -2575,145 +2575,85 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C56" t="str" xml:space="preserve">
-        <v xml:space="preserve">_x000d_
-Each Trail Symbol that lands during the base game will fly into corresponding colored fortune pouch._x000d_
-Any Trail Symbol may trigger the corresponding fortune pouch._x000d_
-More than one fortune pouch can be triggered on a single spin._x000d_
-If fortune pouch(s) are triggered, the corresponding feature will start._x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-The Accumulation of Trail Symbols over time in the BLUE, RED and GREEN fortune pouches have no_x000d_
+        <v xml:space="preserve">
+Each Trail Symbol that lands during the base game will fly into corresponding colored fortune pouch.
+Any Trail Symbol may trigger the corresponding fortune pouch.
+More than one fortune pouch can be triggered on a single spin.
+If fortune pouch(s) are triggered, the corresponding feature will start.
+The Accumulation of Trail Symbols over time in the BLUE, RED and GREEN fortune pouches have no
 effect on triggering the JACKPOT FEATURE or MATSURI FEATURE.</v>
       </c>
       <c r="D56" t="str" xml:space="preserve">
-        <v xml:space="preserve">_x000d_
-Base game에서 획득한 Trail Symbol은 해당 색상의 복주머니로 수집됩니다._x000d_
-Trail Symbol은 해당 복주머니 Feature를 발동할 수 있으며, 하나의 스핀에서 여러 개의 복주머니가 동시에 발동될 수 있습니다._x000d_
-복주머니가 발동되면 해당 Feature가 시작됩니다._x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
+        <v xml:space="preserve">
+Base game에서 획득한 Trail Symbol은 해당 색상의 복주머니로 수집됩니다.
+Trail Symbol은 해당 복주머니 Feature를 발동할 수 있으며, 하나의 스핀에서 여러 개의 복주머니가 동시에 발동될 수 있습니다.
+복주머니가 발동되면 해당 Feature가 시작됩니다.
 파란색, 빨간색, 녹색 복주머니에 누적된 Trail Symbol은 JACKPOT FEATURE 또는 MATSURI FEATURE의 발동 확률에 영향을 주지 않습니다.</v>
       </c>
       <c r="E56" t="str" xml:space="preserve">
-        <v xml:space="preserve">_x000d_
-主游戏期间每个落定的 Trail 符号都会飞入对应颜色的福袋。_x000d_
-任意 Trail 符号都可触发其对应的福袋。_x000d_
-单次旋转中可同时触发多个福袋。_x000d_
-若福袋被触发，对应的功能将随之启动。_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
+        <v xml:space="preserve">
+主游戏期间每个落定的 Trail 符号都会飞入对应颜色的福袋。
+任意 Trail 符号都可触发其对应的福袋。
+单次旋转中可同时触发多个福袋。
+若福袋被触发，对应的功能将随之启动。
 Trail 符号在蓝色、红色和绿色福袋中长期累积，不会影响 JACKPOT FEATURE 或 MATSURI FEATURE 的触发。</v>
       </c>
       <c r="F56" t="str" xml:space="preserve">
-        <v xml:space="preserve">_x000d_
-主遊戲期間每個落定的 Trail 符號都會飛入對應顏色的福袋。_x000d_
-任意 Trail 符號都可觸發其對應的福袋。_x000d_
-單次旋轉中可同時觸發多個福袋。_x000d_
-若福袋被觸發，對應的功能將隨之啟動。_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
+        <v xml:space="preserve">
+主遊戲期間每個落定的 Trail 符號都會飛入對應顏色的福袋。
+任意 Trail 符號都可觸發其對應的福袋。
+單次旋轉中可同時觸發多個福袋。
+若福袋被觸發，對應的功能將隨之啟動。
 Trail 符號在藍色、紅色與綠色福袋中長期累積，不會影響 JACKPOT FEATURE 或 MATSURI FEATURE 的觸發。</v>
       </c>
       <c r="G56" t="str" xml:space="preserve">
-        <v xml:space="preserve">Ang bawat Trail Symbol na lalapag sa base game ay lilipad papunta sa katugmang kulay na fortune pouch._x000d_
-Anumang Trail Symbol ay maaaring mag-trigger ng katugmang fortune pouch._x000d_
-Maaaring ma-trigger ang higit sa isang fortune pouch sa iisang spin._x000d_
-Kapag na-trigger ang (mga) fortune pouch, magsisimula ang katugmang feature._x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
+        <v xml:space="preserve">Ang bawat Trail Symbol na lalapag sa base game ay lilipad papunta sa katugmang kulay na fortune pouch.
+Anumang Trail Symbol ay maaaring mag-trigger ng katugmang fortune pouch.
+Maaaring ma-trigger ang higit sa isang fortune pouch sa iisang spin.
+Kapag na-trigger ang (mga) fortune pouch, magsisimula ang katugmang feature.
 Ang pag-iipon ng mga Trail Symbol sa paglipas ng panahon sa BLUE, RED, at GREEN na fortune pouch ay walang epekto sa pag-trigger ng JACKPOT FEATURE o MATSURI FEATURE.</v>
       </c>
       <c r="H56" t="str" xml:space="preserve">
-        <v xml:space="preserve">_x000d_
-ベースゲーム中に着地した各 Trail シンボルは、対応する色の福袋へ飛び込みます。_x000d_
-いずれの Trail シンボルでも、対応する福袋を発動させることがあります。_x000d_
-1回のスピンで複数の福袋が発動することがあります。_x000d_
-福袋が発動すると、対応するフィーチャーが開始します。_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
+        <v xml:space="preserve">
+ベースゲーム中に着地した各 Trail シンボルは、対応する色の福袋へ飛び込みます。
+いずれの Trail シンボルでも、対応する福袋を発動させることがあります。
+1回のスピンで複数の福袋が発動することがあります。
+福袋が発動すると、対応するフィーチャーが開始します。
 青・赤・緑の福袋に Trail シンボルが時間とともに蓄積されても、JACKPOT FEATURE や MATSURI FEATURE の発動には影響しません。</v>
       </c>
       <c r="I56" t="str" xml:space="preserve">
-        <v xml:space="preserve">_x000d_
-สัญลักษณ์ Trail แต่ละตัวที่ตกลงมาในเกมหลักจะลอยเข้าสู่ถุงนำโชค (fortune pouch) ที่มีสีตรงกัน_x000d_
-สัญลักษณ์ Trail ใด ๆ ก็สามารถกระตุ้นถุงนำโชคที่ตรงกันได้_x000d_
-สามารถกระตุ้นถุงนำโชคได้มากกว่าหนึ่งใบในการหมุนเพียงครั้งเดียว_x000d_
-เมื่อถุงนำโชคถูกกระตุ้น ฟีเจอร์ที่สอดคล้องกันจะเริ่มต้นขึ้น_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
+        <v xml:space="preserve">
+สัญลักษณ์ Trail แต่ละตัวที่ตกลงมาในเกมหลักจะลอยเข้าสู่ถุงนำโชค (fortune pouch) ที่มีสีตรงกัน
+สัญลักษณ์ Trail ใด ๆ ก็สามารถกระตุ้นถุงนำโชคที่ตรงกันได้
+สามารถกระตุ้นถุงนำโชคได้มากกว่าหนึ่งใบในการหมุนเพียงครั้งเดียว
+เมื่อถุงนำโชคถูกกระตุ้น ฟีเจอร์ที่สอดคล้องกันจะเริ่มต้นขึ้น
 การสะสมสัญลักษณ์ Trail เมื่อเวลาผ่านไปในถุงนำโชคสีน้ำเงิน สีแดง และสีเขียว ไม่มีผลต่อการกระตุ้น JACKPOT FEATURE หรือ MATSURI FEATURE</v>
       </c>
       <c r="J56" t="str" xml:space="preserve">
-        <v xml:space="preserve">_x000d_
-Each Trail Symbol that lands during the base game will fly into corresponding colored fortune pouch._x000d_
-Any Trail Symbol may trigger the corresponding fortune pouch._x000d_
-More than one fortune pouch can be triggered on a single spin._x000d_
-If fortune pouch(s) are triggered, the corresponding feature will start._x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-The Accumulation of Trail Symbols over time in the BLUE, RED and GREEN fortune pouches have no_x000d_
+        <v xml:space="preserve">
+Each Trail Symbol that lands during the base game will fly into corresponding colored fortune pouch.
+Any Trail Symbol may trigger the corresponding fortune pouch.
+More than one fortune pouch can be triggered on a single spin.
+If fortune pouch(s) are triggered, the corresponding feature will start.
+The Accumulation of Trail Symbols over time in the BLUE, RED and GREEN fortune pouches have no
 effect on triggering the JACKPOT FEATURE or MATSURI FEATURE.</v>
       </c>
       <c r="K56" t="str" xml:space="preserve">
-        <v xml:space="preserve">_x000d_
-Setiap Trail Symbol yang mendarat semasa base game akan terbang masuk ke dalam fortune pouch yang sewarna dengannya._x000d_
-Mana-mana Trail Symbol boleh mencetuskan fortune pouch yang sepadan._x000d_
-Lebih daripada satu fortune pouch boleh dicetuskan dalam satu spin._x000d_
-Jika fortune pouch dicetuskan, feature yang sepadan akan bermula._x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-Pengumpulan Trail Symbol dari masa ke masa dalam fortune pouch BIRU, MERAH dan HIJAU tidak_x000d_
+        <v xml:space="preserve">
+Setiap Trail Symbol yang mendarat semasa base game akan terbang masuk ke dalam fortune pouch yang sewarna dengannya.
+Mana-mana Trail Symbol boleh mencetuskan fortune pouch yang sepadan.
+Lebih daripada satu fortune pouch boleh dicetuskan dalam satu spin.
+Jika fortune pouch dicetuskan, feature yang sepadan akan bermula.
+Pengumpulan Trail Symbol dari masa ke masa dalam fortune pouch BIRU, MERAH dan HIJAU tidak
 memberi kesan kepada pencetusan JACKPOT FEATURE atau MATSURI FEATURE.</v>
       </c>
       <c r="L56" t="str" xml:space="preserve">
-        <v xml:space="preserve">_x000d_
-Mọi Trail Symbol xuất hiện trong base game sẽ bay vào túi phúc (fortune pouch) cùng màu tương ứng._x000d_
-Bất kỳ Trail Symbol nào cũng có thể kích hoạt túi phúc tương ứng._x000d_
-Có thể kích hoạt nhiều hơn một túi phúc trong cùng một lượt quay._x000d_
-Khi túi phúc được kích hoạt, feature tương ứng sẽ bắt đầu._x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-_x000d_
-Việc tích lũy Trail Symbol theo thời gian trong các túi phúc XANH DƯƠNG, ĐỎ và XANH LÁ không_x000d_
+        <v xml:space="preserve">
+Mọi Trail Symbol xuất hiện trong base game sẽ bay vào túi phúc (fortune pouch) cùng màu tương ứng.
+Bất kỳ Trail Symbol nào cũng có thể kích hoạt túi phúc tương ứng.
+Có thể kích hoạt nhiều hơn một túi phúc trong cùng một lượt quay.
+Khi túi phúc được kích hoạt, feature tương ứng sẽ bắt đầu.
+Việc tích lũy Trail Symbol theo thời gian trong các túi phúc XANH DƯƠNG, ĐỎ và XANH LÁ không
 ảnh hưởng đến việc kích hoạt JACKPOT FEATURE hay MATSURI FEATURE.</v>
       </c>
     </row>
@@ -2763,7 +2703,7 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C58" t="str" xml:space="preserve">
-        <v xml:space="preserve">Any Red Trail Symbol landing in the Red fortune pouch. May trigger the_x000d_
+        <v xml:space="preserve">Any Red Trail Symbol landing in the Red fortune pouch. May trigger the
 JACKPOT FEATURE</v>
       </c>
       <c r="D58" t="str">
@@ -2785,15 +2725,15 @@
         <v>สัญลักษณ์ Red Trail ใด ๆ ที่ตกลงในถุงนำโชคสีแดง อาจกระตุ้น JACKPOT FEATURE ได้</v>
       </c>
       <c r="J58" t="str" xml:space="preserve">
-        <v xml:space="preserve">Any Red Trail Symbol landing in the Red fortune pouch. May trigger the_x000d_
+        <v xml:space="preserve">Any Red Trail Symbol landing in the Red fortune pouch. May trigger the
 JACKPOT FEATURE</v>
       </c>
       <c r="K58" t="str" xml:space="preserve">
-        <v xml:space="preserve">Mana-mana Red Trail Symbol yang mendarat dalam fortune pouch Merah boleh mencetuskan_x000d_
+        <v xml:space="preserve">Mana-mana Red Trail Symbol yang mendarat dalam fortune pouch Merah boleh mencetuskan
 JACKPOT FEATURE</v>
       </c>
       <c r="L58" t="str" xml:space="preserve">
-        <v xml:space="preserve">Bất kỳ Red Trail Symbol nào rơi vào túi phúc Đỏ đều có thể kích hoạt_x000d_
+        <v xml:space="preserve">Bất kỳ Red Trail Symbol nào rơi vào túi phúc Đỏ đều có thể kích hoạt
 JACKPOT FEATURE</v>
       </c>
     </row>
@@ -2805,57 +2745,57 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C59" t="str" xml:space="preserve">
-        <v xml:space="preserve">15 Symbols will be presented, Symbols are revealed by clicking on them._x000d_
-Symbols will reveal JACKPOT symbol or the UPGRADE symbol. Once 3_x000d_
-matching JACKPOT symbols have been revealed, the corresponding_x000d_
+        <v xml:space="preserve">15 Symbols will be presented, Symbols are revealed by clicking on them.
+Symbols will reveal JACKPOT symbol or the UPGRADE symbol. Once 3
+matching JACKPOT symbols have been revealed, the corresponding
 JACKPOT is awarded.</v>
       </c>
       <c r="D59" t="str" xml:space="preserve">
-        <v xml:space="preserve">총 15개의 심볼이 표시됩니다._x000d_
-각 심볼을 선택하면, JACKPOT 심볼 또는 UPGRADE 심볼이 공개됩니다._x000d_
+        <v xml:space="preserve">총 15개의 심볼이 표시됩니다.
+각 심볼을 선택하면, JACKPOT 심볼 또는 UPGRADE 심볼이 공개됩니다.
 동일한 JACKPOT 심볼 3개를 획득하면 해당 JACKPOT이 지급됩니다.</v>
       </c>
       <c r="E59" t="str" xml:space="preserve">
-        <v xml:space="preserve">将出现 15 个符号，点击符号即可揭示其内容。_x000d_
-符号会揭示出 JACKPOT 符号或 UPGRADE 符号。_x000d_
+        <v xml:space="preserve">将出现 15 个符号，点击符号即可揭示其内容。
+符号会揭示出 JACKPOT 符号或 UPGRADE 符号。
 一旦揭示出 3 个相同的 JACKPOT 符号，即可获得对应的 JACKPOT。</v>
       </c>
       <c r="F59" t="str" xml:space="preserve">
-        <v xml:space="preserve">將出現 15 個符號，點擊符號即可揭示其內容。_x000d_
-符號會揭示出 JACKPOT 符號或 UPGRADE 符號。_x000d_
+        <v xml:space="preserve">將出現 15 個符號，點擊符號即可揭示其內容。
+符號會揭示出 JACKPOT 符號或 UPGRADE 符號。
 一旦揭示出 3 個相同的 JACKPOT 符號，即可獲得對應的 JACKPOT。</v>
       </c>
       <c r="G59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Magpapakita ng 15 Simbolo, at makikita ang mga Simbolo sa pamamagitan ng pag-click sa mga ito._x000d_
-Magpapakita ang mga Simbolo ng JACKPOT symbol o UPGRADE symbol._x000d_
+        <v xml:space="preserve">Magpapakita ng 15 Simbolo, at makikita ang mga Simbolo sa pamamagitan ng pag-click sa mga ito.
+Magpapakita ang mga Simbolo ng JACKPOT symbol o UPGRADE symbol.
 Kapag nakapagpakita na ng 3 magkatugmang JACKPOT symbol, igagawad ang kaukulang JACKPOT.</v>
       </c>
       <c r="H59" t="str" xml:space="preserve">
-        <v xml:space="preserve">15 個のシンボルが表示され、クリックすると内容が公開されます。_x000d_
-シンボルからは JACKPOT シンボルまたは UPGRADE シンボルが現れます。_x000d_
+        <v xml:space="preserve">15 個のシンボルが表示され、クリックすると内容が公開されます。
+シンボルからは JACKPOT シンボルまたは UPGRADE シンボルが現れます。
 同じ JACKPOT シンボルが 3 個公開されると、対応する JACKPOT が獲得できます。</v>
       </c>
       <c r="I59" t="str" xml:space="preserve">
-        <v xml:space="preserve">จะมีสัญลักษณ์ปรากฏ 15 ตัว โดยจะเปิดเผยสัญลักษณ์ด้วยการคลิกที่สัญลักษณ์นั้น_x000d_
-สัญลักษณ์จะเผยให้เห็น JACKPOT symbol หรือ UPGRADE symbol_x000d_
+        <v xml:space="preserve">จะมีสัญลักษณ์ปรากฏ 15 ตัว โดยจะเปิดเผยสัญลักษณ์ด้วยการคลิกที่สัญลักษณ์นั้น
+สัญลักษณ์จะเผยให้เห็น JACKPOT symbol หรือ UPGRADE symbol
 เมื่อเปิดเผย JACKPOT symbol ที่ตรงกันครบ 3 ตัว จะได้รับ JACKPOT ที่สอดคล้องกัน</v>
       </c>
       <c r="J59" t="str" xml:space="preserve">
-        <v xml:space="preserve">15 Symbols will be presented, Symbols are revealed by clicking on them._x000d_
-Symbols will reveal JACKPOT symbol or the UPGRADE symbol. Once 3_x000d_
-matching JACKPOT symbols have been revealed, the corresponding_x000d_
+        <v xml:space="preserve">15 Symbols will be presented, Symbols are revealed by clicking on them.
+Symbols will reveal JACKPOT symbol or the UPGRADE symbol. Once 3
+matching JACKPOT symbols have been revealed, the corresponding
 JACKPOT is awarded.</v>
       </c>
       <c r="K59" t="str" xml:space="preserve">
-        <v xml:space="preserve">15 Simbol akan dipaparkan, dan simbol didedahkan dengan mengklik padanya._x000d_
-Simbol akan mendedahkan JACKPOT symbol atau UPGRADE symbol. Sebaik sahaja 3_x000d_
-JACKPOT symbol yang sepadan didedahkan, JACKPOT yang berkenaan_x000d_
+        <v xml:space="preserve">15 Simbol akan dipaparkan, dan simbol didedahkan dengan mengklik padanya.
+Simbol akan mendedahkan JACKPOT symbol atau UPGRADE symbol. Sebaik sahaja 3
+JACKPOT symbol yang sepadan didedahkan, JACKPOT yang berkenaan
 akan dianugerahkan.</v>
       </c>
       <c r="L59" t="str" xml:space="preserve">
-        <v xml:space="preserve">15 biểu tượng sẽ được hiển thị, nhấp vào từng biểu tượng để mở._x000d_
-Biểu tượng sẽ hiện ra JACKPOT symbol hoặc UPGRADE symbol. Khi đã mở được 3_x000d_
-JACKPOT symbol giống nhau, JACKPOT tương ứng_x000d_
+        <v xml:space="preserve">15 biểu tượng sẽ được hiển thị, nhấp vào từng biểu tượng để mở.
+Biểu tượng sẽ hiện ra JACKPOT symbol hoặc UPGRADE symbol. Khi đã mở được 3
+JACKPOT symbol giống nhau, JACKPOT tương ứng
 sẽ được trao.</v>
       </c>
     </row>
@@ -2867,57 +2807,57 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C60" t="str" xml:space="preserve">
-        <v xml:space="preserve">If 3 UPGRADE symbols are revealed before a JACKPOT is awarded,_x000d_
-the JACKPOT won is upgraded to the next level. If Grand is awarded,_x000d_
-it will be awarded twice. The feature ends when one JACKPOT is_x000d_
+        <v xml:space="preserve">If 3 UPGRADE symbols are revealed before a JACKPOT is awarded,
+the JACKPOT won is upgraded to the next level. If Grand is awarded,
+it will be awarded twice. The feature ends when one JACKPOT is
 awarded to the player.</v>
       </c>
       <c r="D60" t="str" xml:space="preserve">
-        <v xml:space="preserve">JACKPOT이 지급되기 전에 UPGRADE 심볼 3개를 획득하면, 획득 예정인 JACPOT이 다음 등급으로 업그레이드 됩니다._x000d_
-GRAND JACKPOT이 당첨된 상태에서 UPGRADE가 적용될 경우, GRAND JACKPOT 보상이 한 번 더 지급됩니다._x000d_
+        <v xml:space="preserve">JACKPOT이 지급되기 전에 UPGRADE 심볼 3개를 획득하면, 획득 예정인 JACPOT이 다음 등급으로 업그레이드 됩니다.
+GRAND JACKPOT이 당첨된 상태에서 UPGRADE가 적용될 경우, GRAND JACKPOT 보상이 한 번 더 지급됩니다.
 플레이어에게 JACKPOT이 지급되면 해당 Feature 는 종료됩니다.</v>
       </c>
       <c r="E60" t="str" xml:space="preserve">
-        <v xml:space="preserve">若在获得 JACKPOT 之前揭示出 3 个 UPGRADE 符号，所赢得的 JACKPOT 将升级至下一等级。_x000d_
-若获得的是 Grand，则会被授予两次。_x000d_
+        <v xml:space="preserve">若在获得 JACKPOT 之前揭示出 3 个 UPGRADE 符号，所赢得的 JACKPOT 将升级至下一等级。
+若获得的是 Grand，则会被授予两次。
 当玩家获得一个 JACKPOT 时，该功能结束。</v>
       </c>
       <c r="F60" t="str" xml:space="preserve">
-        <v xml:space="preserve">若在獲得 JACKPOT 之前揭示出 3 個 UPGRADE 符號，所贏得的 JACKPOT 將升級至下一等級。_x000d_
-若獲得的是 Grand，則會被授予兩次。_x000d_
+        <v xml:space="preserve">若在獲得 JACKPOT 之前揭示出 3 個 UPGRADE 符號，所贏得的 JACKPOT 將升級至下一等級。
+若獲得的是 Grand，則會被授予兩次。
 當玩家獲得一個 JACKPOT 時，該功能結束。</v>
       </c>
       <c r="G60" t="str" xml:space="preserve">
-        <v xml:space="preserve">Kung 3 UPGRADE symbol ang maipakita bago igawad ang isang JACKPOT, ang nanalong JACKPOT ay maa-upgrade sa susunod na antas._x000d_
-Kung Grand ang igawad, igagawad ito nang dalawang beses._x000d_
+        <v xml:space="preserve">Kung 3 UPGRADE symbol ang maipakita bago igawad ang isang JACKPOT, ang nanalong JACKPOT ay maa-upgrade sa susunod na antas.
+Kung Grand ang igawad, igagawad ito nang dalawang beses.
 Magtatapos ang feature kapag naigawad na sa manlalaro ang isang JACKPOT.</v>
       </c>
       <c r="H60" t="str" xml:space="preserve">
-        <v xml:space="preserve">JACKPOT が獲得される前に UPGRADE シンボルが 3 個公開された場合、獲得する JACKPOT は次のレベルにアップグレードされます。_x000d_
-Grand を獲得した場合は、2 回分が付与されます。_x000d_
+        <v xml:space="preserve">JACKPOT が獲得される前に UPGRADE シンボルが 3 個公開された場合、獲得する JACKPOT は次のレベルにアップグレードされます。
+Grand を獲得した場合は、2 回分が付与されます。
 プレイヤーに 1 つの JACKPOT が付与されると、フィーチャーは終了します。</v>
       </c>
       <c r="I60" t="str" xml:space="preserve">
-        <v xml:space="preserve">หากเปิดเผย UPGRADE symbol ครบ 3 ตัวก่อนที่จะได้รับ JACKPOT รางวัล JACKPOT ที่ชนะจะถูกอัปเกรดเป็นระดับถัดไป_x000d_
-หากได้รับ Grand จะมอบรางวัลให้สองครั้ง_x000d_
+        <v xml:space="preserve">หากเปิดเผย UPGRADE symbol ครบ 3 ตัวก่อนที่จะได้รับ JACKPOT รางวัล JACKPOT ที่ชนะจะถูกอัปเกรดเป็นระดับถัดไป
+หากได้รับ Grand จะมอบรางวัลให้สองครั้ง
 ฟีเจอร์จะสิ้นสุดลงเมื่อผู้เล่นได้รับ JACKPOT หนึ่งรายการ</v>
       </c>
       <c r="J60" t="str" xml:space="preserve">
-        <v xml:space="preserve">If 3 UPGRADE symbols are revealed before a JACKPOT is awarded,_x000d_
-the JACKPOT won is upgraded to the next level. If Grand is awarded,_x000d_
-it will be awarded twice. The feature ends when one JACKPOT is_x000d_
+        <v xml:space="preserve">If 3 UPGRADE symbols are revealed before a JACKPOT is awarded,
+the JACKPOT won is upgraded to the next level. If Grand is awarded,
+it will be awarded twice. The feature ends when one JACKPOT is
 awarded to the player.</v>
       </c>
       <c r="K60" t="str" xml:space="preserve">
-        <v xml:space="preserve">Jika 3 UPGRADE symbol didedahkan sebelum JACKPOT dianugerahkan,_x000d_
-JACKPOT yang dimenangi akan dinaik taraf ke tahap seterusnya. Jika Grand dianugerahkan,_x000d_
-ia akan dianugerahkan dua kali. Feature ini tamat apabila satu JACKPOT_x000d_
+        <v xml:space="preserve">Jika 3 UPGRADE symbol didedahkan sebelum JACKPOT dianugerahkan,
+JACKPOT yang dimenangi akan dinaik taraf ke tahap seterusnya. Jika Grand dianugerahkan,
+ia akan dianugerahkan dua kali. Feature ini tamat apabila satu JACKPOT
 dianugerahkan kepada pemain.</v>
       </c>
       <c r="L60" t="str" xml:space="preserve">
-        <v xml:space="preserve">Nếu mở được 3 UPGRADE symbol trước khi một JACKPOT được trao,_x000d_
-JACKPOT giành được sẽ được nâng lên cấp tiếp theo. Nếu Grand được trao,_x000d_
-phần thưởng sẽ được trao hai lần. Feature kết thúc khi người chơi_x000d_
+        <v xml:space="preserve">Nếu mở được 3 UPGRADE symbol trước khi một JACKPOT được trao,
+JACKPOT giành được sẽ được nâng lên cấp tiếp theo. Nếu Grand được trao,
+phần thưởng sẽ được trao hai lần. Feature kết thúc khi người chơi
 được trao một JACKPOT.</v>
       </c>
     </row>
@@ -3043,43 +2983,43 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C64" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Yellow Sticky Symbol     Green Sticky Symbol</v>
       </c>
       <c r="D64" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Yellow Sticky Symbol     Green Sticky Symbol</v>
       </c>
       <c r="E64" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 黄色粘性符号     绿色粘性符号</v>
       </c>
       <c r="F64" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 黃色黏性符號     綠色黏性符號</v>
       </c>
       <c r="G64" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Yellow Sticky Symbol     Green Sticky Symbol</v>
       </c>
       <c r="H64" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 イエロー スティッキー シンボル     グリーン スティッキー シンボル</v>
       </c>
       <c r="I64" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 สัญลักษณ์ Sticky สีเหลือง     สัญลักษณ์ Sticky สีเขียว</v>
       </c>
       <c r="J64" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Yellow Sticky Symbol     Green Sticky Symbol</v>
       </c>
       <c r="K64" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Simbol Sticky Kuning     Simbol Sticky Hijau</v>
       </c>
       <c r="L64" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Biểu tượng Sticky Vàng     Biểu tượng Sticky Xanh</v>
       </c>
     </row>
@@ -3091,133 +3031,107 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C65" t="str" xml:space="preserve">
-        <v xml:space="preserve">If Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri, or Ultimate Matsuri is_x000d_
-triggered, then the Matsuri Feature is triggered. If the Matsuri Feature was triggered from the Mighty Matsuri or the_x000d_
-Ultra Matsuri, the grid will be 5x3 and 3 spins are awarded. Additionally, 6 Yellow Sticky Symbols will be placed on random_x000d_
-positions at the start of the feature._x000d_
-_x000d_
-If the Matsuri Feature was triggered from the Mega Matsuri or the Supreme Matsuri, the grid will be 5x4 and 3_x000d_
-spins are awarded. Additionally, 8 Yellow Symbols will be placed on random positions at the start of the feature._x000d_
-_x000d_
-If the Matsuri Feature was triggered from the Super Matsuri or the Ultimate Matsuri, the grid will be 5x5 and 3_x000d_
-spins are awarded. Additionally, 10 Yellow Symbols will be placed on random positions at the start of the feature._x000d_
-_x000d_
+        <v xml:space="preserve">If Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri, or Ultimate Matsuri is
+triggered, then the Matsuri Feature is triggered. If the Matsuri Feature was triggered from the Mighty Matsuri or the
+Ultra Matsuri, the grid will be 5x3 and 3 spins are awarded. Additionally, 6 Yellow Sticky Symbols will be placed on random
+positions at the start of the feature.
+If the Matsuri Feature was triggered from the Mega Matsuri or the Supreme Matsuri, the grid will be 5x4 and 3
+spins are awarded. Additionally, 8 Yellow Symbols will be placed on random positions at the start of the feature.
+If the Matsuri Feature was triggered from the Super Matsuri or the Ultimate Matsuri, the grid will be 5x5 and 3
+spins are awarded. Additionally, 10 Yellow Symbols will be placed on random positions at the start of the feature.
 &lt;img src="45" width=80 height=80 offset=-20/&gt; and &lt;img src="44" width=80 height=80 offset=-20/&gt; only appears during the Matsuri Feature.</v>
       </c>
       <c r="D65" t="str" xml:space="preserve">
-        <v xml:space="preserve">Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri 또는 Ultimate Matsuri 발동 시 Matsuri Feature가 시작됩니다._x000d_
-Mighty Matsuri 또는 Ultra Matsuri를 통해 진입한 경우, 5×3 그리드와 함께 3회의 스핀이 제공됩니다._x000d_
-Feature 시작 시 6개의 Yellow Sticky Symbol이 무작위 위치에 배치됩니다._x000d_
-_x000d_
-Mega Matsuri 또는 Supreme Matsuri를 통해 Matsuri Feature가 발동된 경우, 5×4 크기의 그리드에서 진행되며 3회의 스핀이 제공됩니다._x000d_
-또한 Feature 시작 시, 8개의  Yellow Sticky Symbol이 무작위 위치에 배치됩니다._x000d_
-_x000d_
-Super Matsuri 또는 Ultimate Matsuri를 통해 진입한 경우, 5×5 그리드와 함께 3회의 스핀이 제공됩니다._x000d_
-Feature 시작 시 10개의 Yellow Sticky Symbol이 무작위 위치에 배치됩니다._x000d_
-_x000d_
+        <v xml:space="preserve">Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri 또는 Ultimate Matsuri 발동 시 Matsuri Feature가 시작됩니다.
+Mighty Matsuri 또는 Ultra Matsuri를 통해 진입한 경우, 5×3 그리드와 함께 3회의 스핀이 제공됩니다.
+Feature 시작 시 6개의 Yellow Sticky Symbol이 무작위 위치에 배치됩니다.
+Mega Matsuri 또는 Supreme Matsuri를 통해 Matsuri Feature가 발동된 경우, 5×4 크기의 그리드에서 진행되며 3회의 스핀이 제공됩니다.
+또한 Feature 시작 시, 8개의  Yellow Sticky Symbol이 무작위 위치에 배치됩니다.
+Super Matsuri 또는 Ultimate Matsuri를 통해 진입한 경우, 5×5 그리드와 함께 3회의 스핀이 제공됩니다.
+Feature 시작 시 10개의 Yellow Sticky Symbol이 무작위 위치에 배치됩니다.
 &lt;img src="45" width=80 height=80 offset=-20/&gt; 및 &lt;img src="44" width=80 height=80 offset=-20/&gt; 심볼은 Matsuri Feature 진행 중에만 등장합니다.</v>
       </c>
       <c r="E65" t="str" xml:space="preserve">
-        <v xml:space="preserve">若触发 Mighty Matsuri、Mega Matsuri、Super Matsuri、Ultra Matsuri、Supreme Matsuri 或 Ultimate Matsuri，则会触发 Matsuri Feature。_x000d_
-若 Matsuri Feature 由 Mighty Matsuri 或 Ultra Matsuri 触发，网格为 5x3，并获得 3 次旋转。_x000d_
-_x000d_
-此外，功能开始时会在随机位置放置 6 个黄色 Sticky 符号。_x000d_
-若 Matsuri Feature 由 Mega Matsuri 或 Supreme Matsuri 触发，网格为 5x4，并获得 3 次旋转。_x000d_
-_x000d_
-此外，功能开始时会在随机位置放置 8 个黄色 Sticky 符号。_x000d_
-若 Matsuri Feature 由 Super Matsuri 或 Ultimate Matsuri 触发，网格为 5x5，并获得 3 次旋转。_x000d_
-_x000d_
-此外，功能开始时会在随机位置放置 10 个黄色 Sticky 符号。_x000d_
-_x000d_
+        <v xml:space="preserve">若触发 Mighty Matsuri、Mega Matsuri、Super Matsuri、Ultra Matsuri、Supreme Matsuri 或 Ultimate Matsuri，则会触发 Matsuri Feature。
+若 Matsuri Feature 由 Mighty Matsuri 或 Ultra Matsuri 触发，网格为 5x3，并获得 3 次旋转。
+此外，功能开始时会在随机位置放置 6 个黄色 Sticky 符号。
+若 Matsuri Feature 由 Mega Matsuri 或 Supreme Matsuri 触发，网格为 5x4，并获得 3 次旋转。
+此外，功能开始时会在随机位置放置 8 个黄色 Sticky 符号。
+若 Matsuri Feature 由 Super Matsuri 或 Ultimate Matsuri 触发，网格为 5x5，并获得 3 次旋转。
+此外，功能开始时会在随机位置放置 10 个黄色 Sticky 符号。
 &lt;img src="45" width=80 height=80 offset=-20/&gt; 与 &lt;img src="44" width=80 height=80 offset=-20/&gt; 仅在 Matsuri Feature 期间出现。</v>
       </c>
       <c r="F65" t="str" xml:space="preserve">
-        <v xml:space="preserve">若觸發 Mighty Matsuri、Mega Matsuri、Super Matsuri、Ultra Matsuri、Supreme Matsuri 或 Ultimate Matsuri，則會觸發 Matsuri Feature。_x000d_
-若 Matsuri Feature 由 Mighty Matsuri 或 Ultra Matsuri 觸發，網格為 5x3，並獲得 3 次旋轉。_x000d_
-_x000d_
-此外，功能開始時會在隨機位置放置 6 個黃色 Sticky 符號。_x000d_
-若 Matsuri Feature 由 Mega Matsuri 或 Supreme Matsuri 觸發，網格為 5x4，並獲得 3 次旋轉。_x000d_
-_x000d_
-此外，功能開始時會在隨機位置放置 8 個黃色 Sticky 符號。_x000d_
-若 Matsuri Feature 由 Super Matsuri 或 Ultimate Matsuri 觸發，網格為 5x5，並獲得 3 次旋轉。_x000d_
-_x000d_
-此外，功能開始時會在隨機位置放置 10 個黃色 Sticky 符號。_x000d_
-_x000d_
+        <v xml:space="preserve">若觸發 Mighty Matsuri、Mega Matsuri、Super Matsuri、Ultra Matsuri、Supreme Matsuri 或 Ultimate Matsuri，則會觸發 Matsuri Feature。
+若 Matsuri Feature 由 Mighty Matsuri 或 Ultra Matsuri 觸發，網格為 5x3，並獲得 3 次旋轉。
+此外，功能開始時會在隨機位置放置 6 個黃色 Sticky 符號。
+若 Matsuri Feature 由 Mega Matsuri 或 Supreme Matsuri 觸發，網格為 5x4，並獲得 3 次旋轉。
+此外，功能開始時會在隨機位置放置 8 個黃色 Sticky 符號。
+若 Matsuri Feature 由 Super Matsuri 或 Ultimate Matsuri 觸發，網格為 5x5，並獲得 3 次旋轉。
+此外，功能開始時會在隨機位置放置 10 個黃色 Sticky 符號。
 &lt;img src="45" width=80 height=80 offset=-20/&gt; 與 &lt;img src="44" width=80 height=80 offset=-20/&gt; 僅在 Matsuri Feature 期間出現。</v>
       </c>
       <c r="G65" t="str" xml:space="preserve">
-        <v xml:space="preserve">Kung ma-trigger ang Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri, o Ultimate Matsuri, mata-trigger ang Matsuri Feature._x000d_
-Kung na-trigger ang Matsuri Feature mula sa Mighty Matsuri o Ultra Matsuri, ang grid ay magiging 5x3 at 3 spins ang igagawad._x000d_
-Bukod pa rito, 6 na Yellow Sticky Symbol ang ilalagay sa mga random na posisyon sa simula ng feature._x000d_
-Kung na-trigger ang Matsuri Feature mula sa Mega Matsuri o Supreme Matsuri, ang grid ay magiging 5x4 at 3 spins ang igagawad._x000d_
-Bukod pa rito, 8 Yellow Sticky Symbol ang ilalagay sa mga random na posisyon sa simula ng feature._x000d_
-Kung na-trigger ang Matsuri Feature mula sa Super Matsuri o Ultimate Matsuri, ang grid ay magiging 5x5 at 3 spins ang igagawad._x000d_
-Bukod pa rito, 10 Yellow Sticky Symbol ang ilalagay sa mga random na posisyon sa simula ng feature._x000d_
-_x000d_
+        <v xml:space="preserve">Kung ma-trigger ang Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri, o Ultimate Matsuri, mata-trigger ang Matsuri Feature.
+Kung na-trigger ang Matsuri Feature mula sa Mighty Matsuri o Ultra Matsuri, ang grid ay magiging 5x3 at 3 spins ang igagawad.
+Bukod pa rito, 6 na Yellow Sticky Symbol ang ilalagay sa mga random na posisyon sa simula ng feature.
+Kung na-trigger ang Matsuri Feature mula sa Mega Matsuri o Supreme Matsuri, ang grid ay magiging 5x4 at 3 spins ang igagawad.
+Bukod pa rito, 8 Yellow Sticky Symbol ang ilalagay sa mga random na posisyon sa simula ng feature.
+Kung na-trigger ang Matsuri Feature mula sa Super Matsuri o Ultimate Matsuri, ang grid ay magiging 5x5 at 3 spins ang igagawad.
+Bukod pa rito, 10 Yellow Sticky Symbol ang ilalagay sa mga random na posisyon sa simula ng feature.
 Lumalabas lang ang &lt;img src="45" width=80 height=80 offset=-20/&gt; at &lt;img src="44" width=80 height=80 offset=-20/&gt; sa panahon ng Matsuri Feature.</v>
       </c>
       <c r="H65" t="str" xml:space="preserve">
-        <v xml:space="preserve">Mighty Matsuri、Mega Matsuri、Super Matsuri、Ultra Matsuri、Supreme Matsuri、または Ultimate Matsuri が発動すると、Matsuri Feature が発動します。_x000d_
-Matsuri Feature が Mighty Matsuri または Ultra Matsuri から発動した場合、グリッドは 5x3 となり、3 回のスピンが付与されます。_x000d_
-さらに、フィーチャー開始時に 6 個のイエロー Sticky シンボルがランダムな位置に配置されます。_x000d_
-Matsuri Feature が Mega Matsuri または Supreme Matsuri から発動した場合、グリッドは 5x4 となり、3 回のスピンが付与されます。_x000d_
-さらに、フィーチャー開始時に 8 個のイエロー Sticky シンボルがランダムな位置に配置されます。_x000d_
-Matsuri Feature が Super Matsuri または Ultimate Matsuri から発動した場合、グリッドは 5x5 となり、3 回のスピンが付与されます。_x000d_
-さらに、フィーチャー開始時に 10 個のイエロー Sticky シンボルがランダムな位置に配置されます。_x000d_
-_x000d_
+        <v xml:space="preserve">Mighty Matsuri、Mega Matsuri、Super Matsuri、Ultra Matsuri、Supreme Matsuri、または Ultimate Matsuri が発動すると、Matsuri Feature が発動します。
+Matsuri Feature が Mighty Matsuri または Ultra Matsuri から発動した場合、グリッドは 5x3 となり、3 回のスピンが付与されます。
+さらに、フィーチャー開始時に 6 個のイエロー Sticky シンボルがランダムな位置に配置されます。
+Matsuri Feature が Mega Matsuri または Supreme Matsuri から発動した場合、グリッドは 5x4 となり、3 回のスピンが付与されます。
+さらに、フィーチャー開始時に 8 個のイエロー Sticky シンボルがランダムな位置に配置されます。
+Matsuri Feature が Super Matsuri または Ultimate Matsuri から発動した場合、グリッドは 5x5 となり、3 回のスピンが付与されます。
+さらに、フィーチャー開始時に 10 個のイエロー Sticky シンボルがランダムな位置に配置されます。
 &lt;img src="45" width=80 height=80 offset=-20/&gt; と &lt;img src="44" width=80 height=80 offset=-20/&gt; は Matsuri Feature 中のみ出現します。</v>
       </c>
       <c r="I65" t="str" xml:space="preserve">
-        <v xml:space="preserve">หากกระตุ้น Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri หรือ Ultimate Matsuri จะเป็นการกระตุ้น Matsuri Feature_x000d_
-หาก Matsuri Feature ถูกกระตุ้นจาก Mighty Matsuri หรือ Ultra Matsuri กริดจะเป็น 5x3 และได้รับ 3 สปิน_x000d_
-นอกจากนี้ จะมีการวาง Yellow Sticky Symbol จำนวน 6 ตัวในตำแหน่งสุ่มเมื่อเริ่มฟีเจอร์_x000d_
-หาก Matsuri Feature ถูกกระตุ้นจาก Mega Matsuri หรือ Supreme Matsuri กริดจะเป็น 5x4 และได้รับ 3 สปิน_x000d_
-นอกจากนี้ จะมีการวาง Yellow Sticky Symbol จำนวน 8 ตัวในตำแหน่งสุ่มเมื่อเริ่มฟีเจอร์_x000d_
-หาก Matsuri Feature ถูกกระตุ้นจาก Super Matsuri หรือ Ultimate Matsuri กริดจะเป็น 5x5 และได้รับ 3 สปิน_x000d_
-นอกจากนี้ จะมีการวาง Yellow Sticky Symbol จำนวน 10 ตัวในตำแหน่งสุ่มเมื่อเริ่มฟีเจอร์_x000d_
-_x000d_
+        <v xml:space="preserve">หากกระตุ้น Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri หรือ Ultimate Matsuri จะเป็นการกระตุ้น Matsuri Feature
+หาก Matsuri Feature ถูกกระตุ้นจาก Mighty Matsuri หรือ Ultra Matsuri กริดจะเป็น 5x3 และได้รับ 3 สปิน
+นอกจากนี้ จะมีการวาง Yellow Sticky Symbol จำนวน 6 ตัวในตำแหน่งสุ่มเมื่อเริ่มฟีเจอร์
+หาก Matsuri Feature ถูกกระตุ้นจาก Mega Matsuri หรือ Supreme Matsuri กริดจะเป็น 5x4 และได้รับ 3 สปิน
+นอกจากนี้ จะมีการวาง Yellow Sticky Symbol จำนวน 8 ตัวในตำแหน่งสุ่มเมื่อเริ่มฟีเจอร์
+หาก Matsuri Feature ถูกกระตุ้นจาก Super Matsuri หรือ Ultimate Matsuri กริดจะเป็น 5x5 และได้รับ 3 สปิน
+นอกจากนี้ จะมีการวาง Yellow Sticky Symbol จำนวน 10 ตัวในตำแหน่งสุ่มเมื่อเริ่มฟีเจอร์
 &lt;img src="45" width=80 height=80 offset=-20/&gt; และ &lt;img src="44" width=80 height=80 offset=-20/&gt; จะปรากฏเฉพาะในระหว่าง Matsuri Feature เท่านั้น</v>
       </c>
       <c r="J65" t="str" xml:space="preserve">
-        <v xml:space="preserve">If Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri, or Ultimate Matsuri is_x000d_
-triggered, then the Matsuri Feature is triggered. If the Matsuri Feature was triggered from the Mighty Matsuri or the_x000d_
-Ultra Matsuri, the grid will be 5x3 and 3 spins are awarded. Additionally, 6 Yellow Sticky Symbols will be placed on random_x000d_
-positions at the start of the feature._x000d_
-_x000d_
-If the Matsuri Feature was triggered from the Mega Matsuri or the Supreme Matsuri, the grid will be 5x4 and 3_x000d_
-spins are awarded. Additionally, 8 Yellow Symbols will be placed on random positions at the start of the feature._x000d_
-_x000d_
-If the Matsuri Feature was triggered from the Super Matsuri or the Ultimate Matsuri, the grid will be 5x5 and 3_x000d_
-spins are awarded. Additionally, 10 Yellow Symbols will be placed on random positions at the start of the feature._x000d_
-_x000d_
+        <v xml:space="preserve">If Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri, or Ultimate Matsuri is
+triggered, then the Matsuri Feature is triggered. If the Matsuri Feature was triggered from the Mighty Matsuri or the
+Ultra Matsuri, the grid will be 5x3 and 3 spins are awarded. Additionally, 6 Yellow Sticky Symbols will be placed on random
+positions at the start of the feature.
+If the Matsuri Feature was triggered from the Mega Matsuri or the Supreme Matsuri, the grid will be 5x4 and 3
+spins are awarded. Additionally, 8 Yellow Symbols will be placed on random positions at the start of the feature.
+If the Matsuri Feature was triggered from the Super Matsuri or the Ultimate Matsuri, the grid will be 5x5 and 3
+spins are awarded. Additionally, 10 Yellow Symbols will be placed on random positions at the start of the feature.
 &lt;img src="45" width=80 height=80 offset=-20/&gt; and &lt;img src="44" width=80 height=80 offset=-20/&gt; only appears during the Matsuri Feature.</v>
       </c>
       <c r="K65" t="str" xml:space="preserve">
-        <v xml:space="preserve">Jika Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri atau Ultimate Matsuri_x000d_
-dicetuskan, maka Matsuri Feature akan dicetuskan. Jika Matsuri Feature dicetuskan daripada Mighty Matsuri atau_x000d_
-Ultra Matsuri, grid akan menjadi 5x3 dan 3 spin dianugerahkan. Selain itu, 6 Yellow Sticky Symbol akan diletakkan pada_x000d_
-kedudukan rawak pada permulaan feature._x000d_
-_x000d_
-Jika Matsuri Feature dicetuskan daripada Mega Matsuri atau Supreme Matsuri, grid akan menjadi 5x4 dan 3_x000d_
-spin dianugerahkan. Selain itu, 8 Yellow Symbol akan diletakkan pada kedudukan rawak pada permulaan feature._x000d_
-_x000d_
-Jika Matsuri Feature dicetuskan daripada Super Matsuri atau Ultimate Matsuri, grid akan menjadi 5x5 dan 3_x000d_
-spin dianugerahkan. Selain itu, 10 Yellow Symbol akan diletakkan pada kedudukan rawak pada permulaan feature._x000d_
-_x000d_
+        <v xml:space="preserve">Jika Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri atau Ultimate Matsuri
+dicetuskan, maka Matsuri Feature akan dicetuskan. Jika Matsuri Feature dicetuskan daripada Mighty Matsuri atau
+Ultra Matsuri, grid akan menjadi 5x3 dan 3 spin dianugerahkan. Selain itu, 6 Yellow Sticky Symbol akan diletakkan pada
+kedudukan rawak pada permulaan feature.
+Jika Matsuri Feature dicetuskan daripada Mega Matsuri atau Supreme Matsuri, grid akan menjadi 5x4 dan 3
+spin dianugerahkan. Selain itu, 8 Yellow Symbol akan diletakkan pada kedudukan rawak pada permulaan feature.
+Jika Matsuri Feature dicetuskan daripada Super Matsuri atau Ultimate Matsuri, grid akan menjadi 5x5 dan 3
+spin dianugerahkan. Selain itu, 10 Yellow Symbol akan diletakkan pada kedudukan rawak pada permulaan feature.
 &lt;img src="45" width=80 height=80 offset=-20/&gt; dan &lt;img src="44" width=80 height=80 offset=-20/&gt; hanya muncul semasa Matsuri Feature.</v>
       </c>
       <c r="L65" t="str" xml:space="preserve">
-        <v xml:space="preserve">Nếu Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri hoặc Ultimate Matsuri được_x000d_
-kích hoạt thì Matsuri Feature sẽ được kích hoạt. Nếu Matsuri Feature được kích hoạt từ Mighty Matsuri hoặc_x000d_
-Ultra Matsuri, lưới sẽ là 5x3 và được trao 3 lượt quay. Ngoài ra, 6 Yellow Sticky Symbol sẽ được đặt ở_x000d_
-các vị trí ngẫu nhiên khi feature bắt đầu._x000d_
-_x000d_
-Nếu Matsuri Feature được kích hoạt từ Mega Matsuri hoặc Supreme Matsuri, lưới sẽ là 5x4 và được trao 3_x000d_
-lượt quay. Ngoài ra, 8 Yellow Symbol sẽ được đặt ở các vị trí ngẫu nhiên khi feature bắt đầu._x000d_
-_x000d_
-Nếu Matsuri Feature được kích hoạt từ Super Matsuri hoặc Ultimate Matsuri, lưới sẽ là 5x5 và được trao 3_x000d_
-lượt quay. Ngoài ra, 10 Yellow Symbol sẽ được đặt ở các vị trí ngẫu nhiên khi feature bắt đầu._x000d_
-_x000d_
+        <v xml:space="preserve">Nếu Mighty Matsuri, Mega Matsuri, Super Matsuri, Ultra Matsuri, Supreme Matsuri hoặc Ultimate Matsuri được
+kích hoạt thì Matsuri Feature sẽ được kích hoạt. Nếu Matsuri Feature được kích hoạt từ Mighty Matsuri hoặc
+Ultra Matsuri, lưới sẽ là 5x3 và được trao 3 lượt quay. Ngoài ra, 6 Yellow Sticky Symbol sẽ được đặt ở
+các vị trí ngẫu nhiên khi feature bắt đầu.
+Nếu Matsuri Feature được kích hoạt từ Mega Matsuri hoặc Supreme Matsuri, lưới sẽ là 5x4 và được trao 3
+lượt quay. Ngoài ra, 8 Yellow Symbol sẽ được đặt ở các vị trí ngẫu nhiên khi feature bắt đầu.
+Nếu Matsuri Feature được kích hoạt từ Super Matsuri hoặc Ultimate Matsuri, lưới sẽ là 5x5 và được trao 3
+lượt quay. Ngoài ra, 10 Yellow Symbol sẽ được đặt ở các vị trí ngẫu nhiên khi feature bắt đầu.
 &lt;img src="45" width=80 height=80 offset=-20/&gt; và &lt;img src="44" width=80 height=80 offset=-20/&gt; chỉ xuất hiện trong Matsuri Feature.</v>
       </c>
     </row>
@@ -3267,43 +3181,43 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C67" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Yellow Sticky Symbol     Green Sticky Symbol</v>
       </c>
       <c r="D67" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Yellow Sticky Symbol     Green Sticky Symbol</v>
       </c>
       <c r="E67" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 黄色粘性符号     绿色粘性符号</v>
       </c>
       <c r="F67" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 黃色黏性符號     綠色黏性符號</v>
       </c>
       <c r="G67" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Yellow Sticky Symbol     Green Sticky Symbol</v>
       </c>
       <c r="H67" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 イエロー スティッキー シンボル     グリーン スティッキー シンボル</v>
       </c>
       <c r="I67" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 สัญลักษณ์ Sticky สีเหลือง     สัญลักษณ์ Sticky สีเขียว</v>
       </c>
       <c r="J67" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Yellow Sticky Symbol     Green Sticky Symbol</v>
       </c>
       <c r="K67" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Simbol Sticky Kuning     Simbol Sticky Hijau</v>
       </c>
       <c r="L67" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Biểu tượng Sticky Vàng     Biểu tượng Sticky Xanh</v>
       </c>
     </row>
@@ -3315,78 +3229,73 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C68" t="str" xml:space="preserve">
-        <v xml:space="preserve">All &lt;img src="45" width=70 height=70 offset=-10/&gt; appearing on screen are held for the remainder of the feature. Positions containing a_x000d_
-held &lt;img src="45" width=70 height=70 offset=-10/&gt; will display a credit prize of x 0.3 - x 50 based on the current bet. If the Matsuri_x000d_
-Feature was triggered from the Ultra Matsuri, Supreme Matsuri, or Ultimate Matsuri, then Mini_x000d_
-or Minor may be displayed instead of a credit prize._x000d_
-_x000d_
-During each Matsuri Feature spin, any &lt;img src="44"width=70 height=70 offset=-10&gt; that lands on screen will award the sum of the awards_x000d_
+        <v xml:space="preserve">All &lt;img src="45" width=70 height=70 offset=-10/&gt; appearing on screen are held for the remainder of the feature. Positions containing a
+held &lt;img src="45" width=70 height=70 offset=-10/&gt; will display a credit prize of x 0.3 - x 50 based on the current bet. If the Matsuri
+Feature was triggered from the Ultra Matsuri, Supreme Matsuri, or Ultimate Matsuri, then Mini
+or Minor may be displayed instead of a credit prize.
+During each Matsuri Feature spin, any &lt;img src="44"width=70 height=70 offset=-10&gt; that lands on screen will award the sum of the awards
 displayed on all &lt;img src="45" width=70 height=70 offset=-10/&gt; and the number of spins remaining is reset to 3.</v>
       </c>
       <c r="D68" t="str" xml:space="preserve">
-        <v xml:space="preserve">화면에 등장한 모든 &lt;img src="45" width=70 height=70 offset=-10/&gt; 심볼은 Feature 종료 시까지 유지됩니다._x000d_
-유지된 &lt;img src="45" width=70 height=70 offset=-10/&gt; 심볼 위치에는 현재 Bet에 따라 x0.3 ~ x50의 Credit Prize가 표시됩니다._x000d_
-Ultra Matsuri, Supreme Matsuri 또는 Ultimate Matsuri를 통해 Matsuri Feature가 발동된 경우, Credit Prize 대신 Mini 또는 Minor Jackpot이 등장할 수 있습니다._x000d_
-_x000d_
-Matsuri Feature 중 &lt;img src="44" width=70 height=70 offset=-10/&gt; 심볼이 등장하면,_x000d_
-모든 &lt;img src="45" width=70 height=70 offset=-10/&gt; 심볼에 표시된 봥의 촘합이 지급 됩니다._x000d_
+        <v xml:space="preserve">화면에 등장한 모든 &lt;img src="45" width=70 height=70 offset=-10/&gt; 심볼은 Feature 종료 시까지 유지됩니다.
+유지된 &lt;img src="45" width=70 height=70 offset=-10/&gt; 심볼 위치에는 현재 Bet에 따라 x0.3 ~ x50의 Credit Prize가 표시됩니다.
+Ultra Matsuri, Supreme Matsuri 또는 Ultimate Matsuri를 통해 Matsuri Feature가 발동된 경우, Credit Prize 대신 Mini 또는 Minor Jackpot이 등장할 수 있습니다.
+Matsuri Feature 중 &lt;img src="44" width=70 height=70 offset=-10/&gt; 심볼이 등장하면,
+모든 &lt;img src="45" width=70 height=70 offset=-10/&gt; 심볼에 표시된 봥의 촘합이 지급 됩니다.
 이후 남은 스핀 수가 3회로 재설정 됩니다.</v>
       </c>
       <c r="E68" t="str" xml:space="preserve">
-        <v xml:space="preserve">屏幕上出现的所有 &lt;img src="45" width=70 height=70 offset=-10/&gt; 将在本功能剩余期间被保留。_x000d_
-包含已保留 &lt;img src="45" width=70 height=70 offset=-10/&gt; 的位置会根据当前投注额显示 x 0.3 – x 50 的金额奖励。_x000d_
-若 Matsuri Feature 由 Ultra Matsuri、Supreme Matsuri 或 Ultimate Matsuri 触发，则可能显示 Mini 或 Minor 以替代金额奖励。_x000d_
+        <v xml:space="preserve">屏幕上出现的所有 &lt;img src="45" width=70 height=70 offset=-10/&gt; 将在本功能剩余期间被保留。
+包含已保留 &lt;img src="45" width=70 height=70 offset=-10/&gt; 的位置会根据当前投注额显示 x 0.3 – x 50 的金额奖励。
+若 Matsuri Feature 由 Ultra Matsuri、Supreme Matsuri 或 Ultimate Matsuri 触发，则可能显示 Mini 或 Minor 以替代金额奖励。
 在每次 Matsuri Feature 旋转中，任意落在屏幕上的 &lt;img src="44" width=70 height=70 offset=-10/&gt; 将赢得所有 &lt;img src="45" width=70 height=70 offset=-10/&gt; 上显示奖励的总和，并将剩余旋转次数重置为 3。</v>
       </c>
       <c r="F68" t="str" xml:space="preserve">
-        <v xml:space="preserve">螢幕上出現的所有 &lt;img src="45" width=70 height=70 offset=-10/&gt; 將在本功能剩餘期間被保留。_x000d_
-包含已保留 &lt;img src="45" width=70 height=70 offset=-10/&gt; 的位置會根據當前投注額顯示 x 0.3 – x 50 的金額獎勵。_x000d_
-若 Matsuri Feature 由 Ultra Matsuri、Supreme Matsuri 或 Ultimate Matsuri 觸發，則可能顯示 Mini 或 Minor 以取代金額獎勵。_x000d_
+        <v xml:space="preserve">螢幕上出現的所有 &lt;img src="45" width=70 height=70 offset=-10/&gt; 將在本功能剩餘期間被保留。
+包含已保留 &lt;img src="45" width=70 height=70 offset=-10/&gt; 的位置會根據當前投注額顯示 x 0.3 – x 50 的金額獎勵。
+若 Matsuri Feature 由 Ultra Matsuri、Supreme Matsuri 或 Ultimate Matsuri 觸發，則可能顯示 Mini 或 Minor 以取代金額獎勵。
 在每次 Matsuri Feature 旋轉中，任意落在螢幕上的 &lt;img src="44" width=70 height=70 offset=-10/&gt; 將贏得所有 &lt;img src="45" width=70 height=70 offset=-10/&gt; 上顯示獎勵的總和，並將剩餘旋轉次數重置為 3。</v>
       </c>
       <c r="G68" t="str" xml:space="preserve">
-        <v xml:space="preserve">Lahat ng &lt;img src="45" width=70 height=70 offset=-10/&gt; na lumalabas sa screen ay hahawakan (held) sa natitirang bahagi ng feature._x000d_
-Ang mga posisyong may hawak na &lt;img src="45" width=70 height=70 offset=-10/&gt; ay magpapakita ng credit prize na x 0.3 – x 50 batay sa kasalukuyang bet._x000d_
-Kung na-trigger ang Matsuri Feature mula sa Ultra Matsuri, Supreme Matsuri, o Ultimate Matsuri, maaaring ipakita ang Mini o Minor sa halip na credit prize._x000d_
+        <v xml:space="preserve">Lahat ng &lt;img src="45" width=70 height=70 offset=-10/&gt; na lumalabas sa screen ay hahawakan (held) sa natitirang bahagi ng feature.
+Ang mga posisyong may hawak na &lt;img src="45" width=70 height=70 offset=-10/&gt; ay magpapakita ng credit prize na x 0.3 – x 50 batay sa kasalukuyang bet.
+Kung na-trigger ang Matsuri Feature mula sa Ultra Matsuri, Supreme Matsuri, o Ultimate Matsuri, maaaring ipakita ang Mini o Minor sa halip na credit prize.
 Sa bawat Matsuri Feature spin, anumang &lt;img src="44" width=70 height=70 offset=-10/&gt; na lalapag sa screen ay magbibigay ng kabuuan ng mga award na nakadisplay sa lahat ng &lt;img src="45" width=70 height=70 offset=-10/&gt;, at ire-reset sa 3 ang bilang ng natitirang spins.</v>
       </c>
       <c r="H68" t="str" xml:space="preserve">
-        <v xml:space="preserve">画面上に出現したすべての &lt;img src="45" width=70 height=70 offset=-10/&gt; は、フィーチャーの残りの間ホールドされます。_x000d_
-ホールドされた &lt;img src="45" width=70 height=70 offset=-10/&gt; を含むポジションには、現在のベットに応じて x 0.3 ～ x 50 のクレジット賞金が表示されます。_x000d_
-Matsuri Feature が Ultra Matsuri、Supreme Matsuri、または Ultimate Matsuri から発動した場合、クレジット賞金の代わりに Mini または Minor が表示されることがあります。_x000d_
+        <v xml:space="preserve">画面上に出現したすべての &lt;img src="45" width=70 height=70 offset=-10/&gt; は、フィーチャーの残りの間ホールドされます。
+ホールドされた &lt;img src="45" width=70 height=70 offset=-10/&gt; を含むポジションには、現在のベットに応じて x 0.3 ～ x 50 のクレジット賞金が表示されます。
+Matsuri Feature が Ultra Matsuri、Supreme Matsuri、または Ultimate Matsuri から発動した場合、クレジット賞金の代わりに Mini または Minor が表示されることがあります。
 各 Matsuri Feature スピン中、画面上に着地したいずれの &lt;img src="44" width=70 height=70 offset=-10/&gt; も、すべての &lt;img src="45" width=70 height=70 offset=-10/&gt; に表示された賞金の合計を獲得し、残りのスピン回数が 3 にリセットされます。</v>
       </c>
       <c r="I68" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=70 height=70 offset=-10/&gt; ทั้งหมดที่ปรากฏบนหน้าจอจะถูกค้างไว้ตลอดช่วงที่เหลือของฟีเจอร์_x000d_
-ตำแหน่งที่มี &lt;img src="45" width=70 height=70 offset=-10/&gt; ที่ถูกค้างไว้จะแสดงรางวัลเครดิต x 0.3 – x 50 โดยอิงตามเดิมพันปัจจุบัน_x000d_
-หาก Matsuri Feature ถูกกระตุ้นจาก Ultra Matsuri, Supreme Matsuri หรือ Ultimate Matsuri อาจแสดง Mini หรือ Minor แทนรางวัลเครดิต_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=70 height=70 offset=-10/&gt; ทั้งหมดที่ปรากฏบนหน้าจอจะถูกค้างไว้ตลอดช่วงที่เหลือของฟีเจอร์
+ตำแหน่งที่มี &lt;img src="45" width=70 height=70 offset=-10/&gt; ที่ถูกค้างไว้จะแสดงรางวัลเครดิต x 0.3 – x 50 โดยอิงตามเดิมพันปัจจุบัน
+หาก Matsuri Feature ถูกกระตุ้นจาก Ultra Matsuri, Supreme Matsuri หรือ Ultimate Matsuri อาจแสดง Mini หรือ Minor แทนรางวัลเครดิต
 ในแต่ละสปินของ Matsuri Feature &lt;img src="44" width=70 height=70 offset=-10/&gt; ใด ๆ ที่ตกลงบนหน้าจอจะมอบผลรวมของรางวัลที่แสดงบน &lt;img src="45" width=70 height=70 offset=-10/&gt; ทั้งหมด และจำนวนสปินที่เหลือจะถูกรีเซ็ตเป็น 3</v>
       </c>
       <c r="J68" t="str" xml:space="preserve">
-        <v xml:space="preserve">All &lt;img src="45" width=70 height=70 offset=-10/&gt; appearing on screen are held for the remainder of the feature. Positions containing a_x000d_
-held &lt;img src="45" width=70 height=70 offset=-10/&gt; will display a credit prize of x 0.3 - x 50 based on the current bet. If the Matsuri_x000d_
-Feature was triggered from the Ultra Matsuri, Supreme Matsuri, or Ultimate Matsuri, then Mini_x000d_
-or Minor may be displayed instead of a credit prize._x000d_
-_x000d_
-During each Matsuri Feature spin, any &lt;img src="44"width=70 height=70 offset=-10&gt; that lands on screen will award the sum of the awards_x000d_
+        <v xml:space="preserve">All &lt;img src="45" width=70 height=70 offset=-10/&gt; appearing on screen are held for the remainder of the feature. Positions containing a
+held &lt;img src="45" width=70 height=70 offset=-10/&gt; will display a credit prize of x 0.3 - x 50 based on the current bet. If the Matsuri
+Feature was triggered from the Ultra Matsuri, Supreme Matsuri, or Ultimate Matsuri, then Mini
+or Minor may be displayed instead of a credit prize.
+During each Matsuri Feature spin, any &lt;img src="44"width=70 height=70 offset=-10&gt; that lands on screen will award the sum of the awards
 displayed on all &lt;img src="45" width=70 height=70 offset=-10/&gt; and the number of spins remaining is reset to 3.</v>
       </c>
       <c r="K68" t="str" xml:space="preserve">
-        <v xml:space="preserve">Semua &lt;img src="45" width=70 height=70 offset=-10/&gt; yang muncul pada skrin akan ditahan sepanjang baki feature. Kedudukan yang mengandungi_x000d_
-&lt;img src="45" width=70 height=70 offset=-10/&gt; yang ditahan akan memaparkan hadiah kredit x 0.3 - x 50 berdasarkan pusta semasa. Jika Matsuri_x000d_
-Feature dicetuskan daripada Ultra Matsuri, Supreme Matsuri atau Ultimate Matsuri, maka Mini_x000d_
-atau Minor mungkin dipaparkan sebagai ganti hadiah kredit._x000d_
-_x000d_
-Semasa setiap spin Matsuri Feature, mana-mana &lt;img src="44" width=70 height=70 offset=-10/&gt; yang mendarat pada skrin akan menganugerahkan jumlah keseluruhan_x000d_
+        <v xml:space="preserve">Semua &lt;img src="45" width=70 height=70 offset=-10/&gt; yang muncul pada skrin akan ditahan sepanjang baki feature. Kedudukan yang mengandungi
+&lt;img src="45" width=70 height=70 offset=-10/&gt; yang ditahan akan memaparkan hadiah kredit x 0.3 - x 50 berdasarkan pusta semasa. Jika Matsuri
+Feature dicetuskan daripada Ultra Matsuri, Supreme Matsuri atau Ultimate Matsuri, maka Mini
+atau Minor mungkin dipaparkan sebagai ganti hadiah kredit.
+Semasa setiap spin Matsuri Feature, mana-mana &lt;img src="44" width=70 height=70 offset=-10/&gt; yang mendarat pada skrin akan menganugerahkan jumlah keseluruhan
 hadiah yang dipaparkan pada semua &lt;img src="45" width=70 height=70 offset=-10/&gt; dan bilangan spin yang berbaki akan ditetapkan semula kepada 3.</v>
       </c>
       <c r="L68" t="str" xml:space="preserve">
-        <v xml:space="preserve">Tất cả &lt;img src="45" width=70 height=70 offset=-10/&gt; xuất hiện trên màn hình sẽ được giữ lại trong suốt thời gian còn lại của feature. Các vị trí chứa_x000d_
-&lt;img src="45" width=70 height=70 offset=-10/&gt; được giữ lại sẽ hiển thị giải thưởng tín dụng từ x 0.3 - x 50 dựa trên mức cược hiện tại. Nếu Matsuri_x000d_
-Feature được kích hoạt từ Ultra Matsuri, Supreme Matsuri hoặc Ultimate Matsuri thì Mini_x000d_
-hoặc Minor có thể được hiển thị thay cho giải thưởng tín dụng._x000d_
-_x000d_
-Trong mỗi lượt quay của Matsuri Feature, bất kỳ &lt;img src="44" width=70 height=70 offset=-10/&gt; nào rơi trên màn hình sẽ trao tổng các giải thưởng_x000d_
+        <v xml:space="preserve">Tất cả &lt;img src="45" width=70 height=70 offset=-10/&gt; xuất hiện trên màn hình sẽ được giữ lại trong suốt thời gian còn lại của feature. Các vị trí chứa
+&lt;img src="45" width=70 height=70 offset=-10/&gt; được giữ lại sẽ hiển thị giải thưởng tín dụng từ x 0.3 - x 50 dựa trên mức cược hiện tại. Nếu Matsuri
+Feature được kích hoạt từ Ultra Matsuri, Supreme Matsuri hoặc Ultimate Matsuri thì Mini
+hoặc Minor có thể được hiển thị thay cho giải thưởng tín dụng.
+Trong mỗi lượt quay của Matsuri Feature, bất kỳ &lt;img src="44" width=70 height=70 offset=-10/&gt; nào rơi trên màn hình sẽ trao tổng các giải thưởng
 được hiển thị trên tất cả &lt;img src="45" width=70 height=70 offset=-10/&gt;, và số lượt quay còn lại được đặt lại thành 3.</v>
       </c>
     </row>
@@ -3436,43 +3345,43 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C70" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Yellow Sticky Symbol     Green Sticky Symbol</v>
       </c>
       <c r="D70" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Yellow Sticky Symbol     Green Sticky Symbol</v>
       </c>
       <c r="E70" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 黄色粘性符号     绿色粘性符号</v>
       </c>
       <c r="F70" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 黃色黏性符號     綠色黏性符號</v>
       </c>
       <c r="G70" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Yellow Sticky Symbol     Green Sticky Symbol</v>
       </c>
       <c r="H70" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 イエロー スティッキー シンボル     グリーン スティッキー シンボル</v>
       </c>
       <c r="I70" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 สัญลักษณ์ Sticky สีเหลือง     สัญลักษณ์ Sticky สีเขียว</v>
       </c>
       <c r="J70" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Yellow Sticky Symbol     Green Sticky Symbol</v>
       </c>
       <c r="K70" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Simbol Sticky Kuning     Simbol Sticky Hijau</v>
       </c>
       <c r="L70" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;_x000d_
+        <v xml:space="preserve">&lt;img src="45" width=180 height=180/&gt;           &lt;img src="44" width=180 height=180/&gt;
 Biểu tượng Sticky Vàng     Biểu tượng Sticky Xanh</v>
       </c>
     </row>
@@ -3484,115 +3393,105 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C71" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; are evaluated when they land on screen. If multiple &lt;img src="44" width=60 height=60 offset=-7/&gt; land on screen, they are evaluated_x000d_
-one at a time. Before a &lt;img src="44" width=60 height=60 offset=-7/&gt; is evaluated, all previously evaluated &lt;img src="44" width=60 height=60 offset=-7/&gt; will transform into &lt;img src="45" width=60 height=60 offset=-7/&gt;._x000d_
-_x000d_
-Remaining spins will be played only if there are positions that do not contain &lt;img src="45" width=60 height=60 offset=-7/&gt; nor &lt;img src="44" width=60 height=60 offset=-7/&gt;. If all_x000d_
-positions are held, the value displayed in the GRAND jackpot meter is awarded._x000d_
-_x000d_
-An alternate set of reels is used during the Matsuri Feature. All symbols appearing on the reels_x000d_
-except for &lt;img src="45" width=60 height=60 offset=-7/&gt; and &lt;img src="44" width=60 height=60 offset=-7/&gt; are grayed out and not evaluated. The distribution of prizes changes_x000d_
+        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; are evaluated when they land on screen. If multiple &lt;img src="44" width=60 height=60 offset=-7/&gt; land on screen, they are evaluated
+one at a time. Before a &lt;img src="44" width=60 height=60 offset=-7/&gt; is evaluated, all previously evaluated &lt;img src="44" width=60 height=60 offset=-7/&gt; will transform into &lt;img src="45" width=60 height=60 offset=-7/&gt;.
+Remaining spins will be played only if there are positions that do not contain &lt;img src="45" width=60 height=60 offset=-7/&gt; nor &lt;img src="44" width=60 height=60 offset=-7/&gt;. If all
+positions are held, the value displayed in the GRAND jackpot meter is awarded.
+An alternate set of reels is used during the Matsuri Feature. All symbols appearing on the reels
+except for &lt;img src="45" width=60 height=60 offset=-7/&gt; and &lt;img src="44" width=60 height=60 offset=-7/&gt; are grayed out and not evaluated. The distribution of prizes changes
 with bet option. Credit prizes appearing on screen are awarded as shown.</v>
       </c>
       <c r="D71" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; 심볼은 등장 시 즉시 평가됩니다._x000d_
-여러 개의 &lt;img src="44" width=60 height=60 offset=-7/&gt; 심볼이 등장한 경우 순차적으로 평가되며,_x000d_
-평가가 완료된 &lt;img src="44" width=60 height=60 offset=-7/&gt; 심볼은 &lt;img src="45" width=60 height=60 offset=-7/&gt; 심볼로 변환됩니다._x000d_
-_x000d_
-&lt;img src="45" width=60 height=60 offset=-7/&gt; 또는 &lt;img src="44" width=60 height=60 offset=-7/&gt; 심볼이 없는 빈 위치가 남아 있는 경우에만 추가 스핀이 진행됩니다._x000d_
-모든 위치가 채워지면 GRAND Jackpot 금액이 지급됩니다._x000d_
-_x000d_
-Matsuri Feature에서는 전용 Reel Set이 사용되며,_x000d_
-&lt;img src="45" width=60 height=60 offset=-7/&gt; 및 &lt;img src="44" width=60 height=60 offset=-7/&gt;을 제외한 모든 심볼은 회색으로 표시되고 평가되지 않습니다._x000d_
-보상 분포는 Bet 옵션에 따라 달라지며,_x000d_
+        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; 심볼은 등장 시 즉시 평가됩니다.
+여러 개의 &lt;img src="44" width=60 height=60 offset=-7/&gt; 심볼이 등장한 경우 순차적으로 평가되며,
+평가가 완료된 &lt;img src="44" width=60 height=60 offset=-7/&gt; 심볼은 &lt;img src="45" width=60 height=60 offset=-7/&gt; 심볼로 변환됩니다.
+&lt;img src="45" width=60 height=60 offset=-7/&gt; 또는 &lt;img src="44" width=60 height=60 offset=-7/&gt; 심볼이 없는 빈 위치가 남아 있는 경우에만 추가 스핀이 진행됩니다.
+모든 위치가 채워지면 GRAND Jackpot 금액이 지급됩니다.
+Matsuri Feature에서는 전용 Reel Set이 사용되며,
+&lt;img src="45" width=60 height=60 offset=-7/&gt; 및 &lt;img src="44" width=60 height=60 offset=-7/&gt;을 제외한 모든 심볼은 회색으로 표시되고 평가되지 않습니다.
+보상 분포는 Bet 옵션에 따라 달라지며,
 화면에 표시된 Credit Prize는 그대로 지급됩니다.</v>
       </c>
       <c r="E71" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; 在落到屏幕上时进行结算。_x000d_
-若多个 &lt;img src="44" width=60 height=60 offset=-7/&gt; 同时落在屏幕上，将逐一结算。_x000d_
-在结算某个 &lt;img src="44" width=60 height=60 offset=-7/&gt; 之前，所有此前已结算的 &lt;img src="44" width=60 height=60 offset=-7/&gt; 都会转变为 &lt;img src="45" width=60 height=60 offset=-7/&gt;。_x000d_
-仅当存在既不含 &lt;img src="45" width=60 height=60 offset=-7/&gt; 也不含 &lt;img src="44" width=60 height=60 offset=-7/&gt; 的位置时，才会进行剩余的旋转。_x000d_
-若所有位置均被保留，则授予 GRAND 累积奖池计量表中显示的数值。_x000d_
-Matsuri Feature 期间使用另一套卷轴。_x000d_
-卷轴上出现的除 &lt;img src="45" width=60 height=60 offset=-7/&gt; 与 &lt;img src="44" width=60 height=60 offset=-7/&gt; 以外的所有符号均会变灰且不参与结算。_x000d_
-奖励的分布会随投注选项而变化。_x000d_
+        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; 在落到屏幕上时进行结算。
+若多个 &lt;img src="44" width=60 height=60 offset=-7/&gt; 同时落在屏幕上，将逐一结算。
+在结算某个 &lt;img src="44" width=60 height=60 offset=-7/&gt; 之前，所有此前已结算的 &lt;img src="44" width=60 height=60 offset=-7/&gt; 都会转变为 &lt;img src="45" width=60 height=60 offset=-7/&gt;。
+仅当存在既不含 &lt;img src="45" width=60 height=60 offset=-7/&gt; 也不含 &lt;img src="44" width=60 height=60 offset=-7/&gt; 的位置时，才会进行剩余的旋转。
+若所有位置均被保留，则授予 GRAND 累积奖池计量表中显示的数值。
+Matsuri Feature 期间使用另一套卷轴。
+卷轴上出现的除 &lt;img src="45" width=60 height=60 offset=-7/&gt; 与 &lt;img src="44" width=60 height=60 offset=-7/&gt; 以外的所有符号均会变灰且不参与结算。
+奖励的分布会随投注选项而变化。
 屏幕上出现的金额奖励将按所示授予。</v>
       </c>
       <c r="F71" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; 在落到螢幕上時進行結算。_x000d_
-若多個 &lt;img src="44" width=60 height=60 offset=-7/&gt; 同時落在螢幕上，將逐一結算。_x000d_
-在結算某個 &lt;img src="44" width=60 height=60 offset=-7/&gt; 之前，所有此前已結算的 &lt;img src="44" width=60 height=60 offset=-7/&gt; 都會轉變為 &lt;img src="45" width=60 height=60 offset=-7/&gt;。_x000d_
-僅當存在既不含 &lt;img src="45" width=60 height=60 offset=-7/&gt; 也不含 &lt;img src="44" width=60 height=60 offset=-7/&gt; 的位置時，才會進行剩餘的旋轉。_x000d_
-若所有位置均被保留，則授予 GRAND 累積獎金計量表中顯示的數值。_x000d_
-Matsuri Feature 期間使用另一套捲軸。_x000d_
-捲軸上出現的除 &lt;img src="45" width=60 height=60 offset=-7/&gt; 與 &lt;img src="44" width=60 height=60 offset=-7/&gt; 以外的所有符號均會變灰且不參與結算。_x000d_
-獎勵的分佈會隨投注選項而變化。_x000d_
+        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; 在落到螢幕上時進行結算。
+若多個 &lt;img src="44" width=60 height=60 offset=-7/&gt; 同時落在螢幕上，將逐一結算。
+在結算某個 &lt;img src="44" width=60 height=60 offset=-7/&gt; 之前，所有此前已結算的 &lt;img src="44" width=60 height=60 offset=-7/&gt; 都會轉變為 &lt;img src="45" width=60 height=60 offset=-7/&gt;。
+僅當存在既不含 &lt;img src="45" width=60 height=60 offset=-7/&gt; 也不含 &lt;img src="44" width=60 height=60 offset=-7/&gt; 的位置時，才會進行剩餘的旋轉。
+若所有位置均被保留，則授予 GRAND 累積獎金計量表中顯示的數值。
+Matsuri Feature 期間使用另一套捲軸。
+捲軸上出現的除 &lt;img src="45" width=60 height=60 offset=-7/&gt; 與 &lt;img src="44" width=60 height=60 offset=-7/&gt; 以外的所有符號均會變灰且不參與結算。
+獎勵的分佈會隨投注選項而變化。
 螢幕上出現的金額獎勵將按所示授予。</v>
       </c>
       <c r="G71" t="str" xml:space="preserve">
-        <v xml:space="preserve">Ang &lt;img src="44" width=60 height=60 offset=-7/&gt; ay ineevaluate kapag lumapag ito sa screen._x000d_
-Kung maraming &lt;img src="44" width=60 height=60 offset=-7/&gt; ang lumapag sa screen, isa-isa silang ieevaluate._x000d_
-Bago ievaluate ang isang &lt;img src="44" width=60 height=60 offset=-7/&gt;, lahat ng dating na-evaluate na &lt;img src="44" width=60 height=60 offset=-7/&gt; ay magtatransform sa &lt;img src="45" width=60 height=60 offset=-7/&gt;._x000d_
-Ang natitirang spins ay laro lamang kung may mga posisyon na walang &lt;img src="45" width=60 height=60 offset=-7/&gt; ni &lt;img src="44" width=60 height=60 offset=-7/&gt;._x000d_
-Kung lahat ng posisyon ay hawak (held), igagawad ang halagang nakadisplay sa GRAND jackpot meter._x000d_
-May ibang set ng reels na ginagamit sa panahon ng Matsuri Feature._x000d_
-Lahat ng simbolong lumalabas sa reels maliban sa &lt;img src="45" width=60 height=60 offset=-7/&gt; at &lt;img src="44" width=60 height=60 offset=-7/&gt; ay ginagawang kulay-abo (grayed out) at hindi ineevaluate._x000d_
-Nagbabago ang distribusyon ng mga premyo ayon sa bet option._x000d_
+        <v xml:space="preserve">Ang &lt;img src="44" width=60 height=60 offset=-7/&gt; ay ineevaluate kapag lumapag ito sa screen.
+Kung maraming &lt;img src="44" width=60 height=60 offset=-7/&gt; ang lumapag sa screen, isa-isa silang ieevaluate.
+Bago ievaluate ang isang &lt;img src="44" width=60 height=60 offset=-7/&gt;, lahat ng dating na-evaluate na &lt;img src="44" width=60 height=60 offset=-7/&gt; ay magtatransform sa &lt;img src="45" width=60 height=60 offset=-7/&gt;.
+Ang natitirang spins ay laro lamang kung may mga posisyon na walang &lt;img src="45" width=60 height=60 offset=-7/&gt; ni &lt;img src="44" width=60 height=60 offset=-7/&gt;.
+Kung lahat ng posisyon ay hawak (held), igagawad ang halagang nakadisplay sa GRAND jackpot meter.
+May ibang set ng reels na ginagamit sa panahon ng Matsuri Feature.
+Lahat ng simbolong lumalabas sa reels maliban sa &lt;img src="45" width=60 height=60 offset=-7/&gt; at &lt;img src="44" width=60 height=60 offset=-7/&gt; ay ginagawang kulay-abo (grayed out) at hindi ineevaluate.
+Nagbabago ang distribusyon ng mga premyo ayon sa bet option.
 Ang mga credit prize na lumalabas sa screen ay igagawad gaya ng ipinapakita.</v>
       </c>
       <c r="H71" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; は画面に着地した時点で評価されます。_x000d_
-複数の &lt;img src="44" width=60 height=60 offset=-7/&gt; が画面に着地した場合は、1 つずつ順番に評価されます。_x000d_
-ある &lt;img src="44" width=60 height=60 offset=-7/&gt; が評価される前に、それまでに評価済みのすべての &lt;img src="44" width=60 height=60 offset=-7/&gt; は &lt;img src="45" width=60 height=60 offset=-7/&gt; に変化します。_x000d_
-残りのスピンは、&lt;img src="45" width=60 height=60 offset=-7/&gt; も &lt;img src="44" width=60 height=60 offset=-7/&gt; も含まないポジションがある場合にのみ行われます。_x000d_
-すべてのポジションがホールドされている場合は、GRAND ジャックポットメーターに表示された値が付与されます。_x000d_
-Matsuri Feature 中は別のリールセットが使用されます。_x000d_
-リール上に出現する &lt;img src="45" width=60 height=60 offset=-7/&gt; と &lt;img src="44" width=60 height=60 offset=-7/&gt; 以外のすべてのシンボルはグレーアウトされ、評価されません。_x000d_
-賞金の分布はベットオプションによって変化します。_x000d_
+        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; は画面に着地した時点で評価されます。
+複数の &lt;img src="44" width=60 height=60 offset=-7/&gt; が画面に着地した場合は、1 つずつ順番に評価されます。
+ある &lt;img src="44" width=60 height=60 offset=-7/&gt; が評価される前に、それまでに評価済みのすべての &lt;img src="44" width=60 height=60 offset=-7/&gt; は &lt;img src="45" width=60 height=60 offset=-7/&gt; に変化します。
+残りのスピンは、&lt;img src="45" width=60 height=60 offset=-7/&gt; も &lt;img src="44" width=60 height=60 offset=-7/&gt; も含まないポジションがある場合にのみ行われます。
+すべてのポジションがホールドされている場合は、GRAND ジャックポットメーターに表示された値が付与されます。
+Matsuri Feature 中は別のリールセットが使用されます。
+リール上に出現する &lt;img src="45" width=60 height=60 offset=-7/&gt; と &lt;img src="44" width=60 height=60 offset=-7/&gt; 以外のすべてのシンボルはグレーアウトされ、評価されません。
+賞金の分布はベットオプションによって変化します。
 画面上に表示されたクレジット賞金は、表示どおりに付与されます。</v>
       </c>
       <c r="I71" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; จะถูกประเมินผลเมื่อตกลงบนหน้าจอ_x000d_
-หากมี &lt;img src="44" width=60 height=60 offset=-7/&gt; หลายตัวตกลงบนหน้าจอ จะถูกประเมินผลทีละตัว_x000d_
-ก่อนที่จะประเมิน &lt;img src="44" width=60 height=60 offset=-7/&gt; ตัวใดตัวหนึ่ง &lt;img src="44" width=60 height=60 offset=-7/&gt; ที่ถูกประเมินผลไปก่อนหน้าทั้งหมดจะแปลงร่างเป็น &lt;img src="45" width=60 height=60 offset=-7/&gt;_x000d_
-สปินที่เหลือจะเล่นก็ต่อเมื่อมีตำแหน่งที่ไม่มีทั้ง &lt;img src="45" width=60 height=60 offset=-7/&gt; และ &lt;img src="44" width=60 height=60 offset=-7/&gt;_x000d_
-หากทุกตำแหน่งถูกค้างไว้ทั้งหมด จะได้รับค่าที่แสดงในมิเตอร์แจ็คพอต GRAND_x000d_
-ในระหว่าง Matsuri Feature จะใช้ชุดรีลอีกชุดหนึ่ง_x000d_
-สัญลักษณ์ทั้งหมดที่ปรากฏบนรีลยกเว้น &lt;img src="45" width=60 height=60 offset=-7/&gt; และ &lt;img src="44" width=60 height=60 offset=-7/&gt; จะถูกทำให้เป็นสีเทาและไม่ถูกประเมินผล_x000d_
-การกระจายของรางวัลจะเปลี่ยนแปลงตามตัวเลือกเดิมพัน_x000d_
+        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; จะถูกประเมินผลเมื่อตกลงบนหน้าจอ
+หากมี &lt;img src="44" width=60 height=60 offset=-7/&gt; หลายตัวตกลงบนหน้าจอ จะถูกประเมินผลทีละตัว
+ก่อนที่จะประเมิน &lt;img src="44" width=60 height=60 offset=-7/&gt; ตัวใดตัวหนึ่ง &lt;img src="44" width=60 height=60 offset=-7/&gt; ที่ถูกประเมินผลไปก่อนหน้าทั้งหมดจะแปลงร่างเป็น &lt;img src="45" width=60 height=60 offset=-7/&gt;
+สปินที่เหลือจะเล่นก็ต่อเมื่อมีตำแหน่งที่ไม่มีทั้ง &lt;img src="45" width=60 height=60 offset=-7/&gt; และ &lt;img src="44" width=60 height=60 offset=-7/&gt;
+หากทุกตำแหน่งถูกค้างไว้ทั้งหมด จะได้รับค่าที่แสดงในมิเตอร์แจ็คพอต GRAND
+ในระหว่าง Matsuri Feature จะใช้ชุดรีลอีกชุดหนึ่ง
+สัญลักษณ์ทั้งหมดที่ปรากฏบนรีลยกเว้น &lt;img src="45" width=60 height=60 offset=-7/&gt; และ &lt;img src="44" width=60 height=60 offset=-7/&gt; จะถูกทำให้เป็นสีเทาและไม่ถูกประเมินผล
+การกระจายของรางวัลจะเปลี่ยนแปลงตามตัวเลือกเดิมพัน
 รางวัลเครดิตที่ปรากฏบนหน้าจอจะได้รับตามที่แสดง</v>
       </c>
       <c r="J71" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; are evaluated when they land on screen. If multiple &lt;img src="44" width=60 height=60 offset=-7/&gt; land on screen, they are evaluated_x000d_
-one at a time. Before a &lt;img src="44" width=60 height=60 offset=-7/&gt; is evaluated, all previously evaluated &lt;img src="44" width=60 height=60 offset=-7/&gt; will transform into &lt;img src="45" width=60 height=60 offset=-7/&gt;._x000d_
-_x000d_
-Remaining spins will be played only if there are positions that do not contain &lt;img src="45" width=60 height=60 offset=-7/&gt; nor &lt;img src="44" width=60 height=60 offset=-7/&gt;. If all_x000d_
-positions are held, the value displayed in the GRAND jackpot meter is awarded._x000d_
-_x000d_
-An alternate set of reels is used during the Matsuri Feature. All symbols appearing on the reels_x000d_
-except for &lt;img src="45" width=60 height=60 offset=-7/&gt; and &lt;img src="44" width=60 height=60 offset=-7/&gt; are grayed out and not evaluated. The distribution of prizes changes_x000d_
+        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; are evaluated when they land on screen. If multiple &lt;img src="44" width=60 height=60 offset=-7/&gt; land on screen, they are evaluated
+one at a time. Before a &lt;img src="44" width=60 height=60 offset=-7/&gt; is evaluated, all previously evaluated &lt;img src="44" width=60 height=60 offset=-7/&gt; will transform into &lt;img src="45" width=60 height=60 offset=-7/&gt;.
+Remaining spins will be played only if there are positions that do not contain &lt;img src="45" width=60 height=60 offset=-7/&gt; nor &lt;img src="44" width=60 height=60 offset=-7/&gt;. If all
+positions are held, the value displayed in the GRAND jackpot meter is awarded.
+An alternate set of reels is used during the Matsuri Feature. All symbols appearing on the reels
+except for &lt;img src="45" width=60 height=60 offset=-7/&gt; and &lt;img src="44" width=60 height=60 offset=-7/&gt; are grayed out and not evaluated. The distribution of prizes changes
 with bet option. Credit prizes appearing on screen are awarded as shown.</v>
       </c>
       <c r="K71" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; dinilai apabila ia mendarat pada skrin. Jika beberapa &lt;img src="44" width=60 height=60 offset=-7/&gt; mendarat pada skrin, ia dinilai_x000d_
-satu demi satu. Sebelum sesuatu &lt;img src="44" width=60 height=60 offset=-7/&gt; dinilai, semua &lt;img src="44" width=60 height=60 offset=-7/&gt; yang telah dinilai sebelum ini akan bertukar menjadi &lt;img src="45" width=60 height=60 offset=-7/&gt;._x000d_
-_x000d_
-Spin yang berbaki hanya akan dimainkan jika terdapat kedudukan yang tidak mengandungi &lt;img src="45" width=60 height=60 offset=-7/&gt; mahupun &lt;img src="44" width=60 height=60 offset=-7/&gt;. Jika semua_x000d_
-kedudukan ditahan, nilai yang dipaparkan pada meter jackpot GRAND akan dianugerahkan._x000d_
-_x000d_
-Set reel yang berbeza digunakan semasa Matsuri Feature. Semua simbol yang muncul pada reel_x000d_
-kecuali &lt;img src="45" width=60 height=60 offset=-7/&gt; dan &lt;img src="44" width=60 height=60 offset=-7/&gt; akan dikelabukan dan tidak dinilai. Pembahagian hadiah berubah_x000d_
+        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; dinilai apabila ia mendarat pada skrin. Jika beberapa &lt;img src="44" width=60 height=60 offset=-7/&gt; mendarat pada skrin, ia dinilai
+satu demi satu. Sebelum sesuatu &lt;img src="44" width=60 height=60 offset=-7/&gt; dinilai, semua &lt;img src="44" width=60 height=60 offset=-7/&gt; yang telah dinilai sebelum ini akan bertukar menjadi &lt;img src="45" width=60 height=60 offset=-7/&gt;.
+Spin yang berbaki hanya akan dimainkan jika terdapat kedudukan yang tidak mengandungi &lt;img src="45" width=60 height=60 offset=-7/&gt; mahupun &lt;img src="44" width=60 height=60 offset=-7/&gt;. Jika semua
+kedudukan ditahan, nilai yang dipaparkan pada meter jackpot GRAND akan dianugerahkan.
+Set reel yang berbeza digunakan semasa Matsuri Feature. Semua simbol yang muncul pada reel
+kecuali &lt;img src="45" width=60 height=60 offset=-7/&gt; dan &lt;img src="44" width=60 height=60 offset=-7/&gt; akan dikelabukan dan tidak dinilai. Pembahagian hadiah berubah
 mengikut pilihan pusta. Hadiah kredit yang muncul pada skrin dianugerahkan seperti yang dipaparkan.</v>
       </c>
       <c r="L71" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; được tính khi rơi trên màn hình. Nếu nhiều &lt;img src="44" width=60 height=60 offset=-7/&gt; cùng rơi trên màn hình, chúng sẽ được tính_x000d_
-lần lượt từng cái một. Trước khi một &lt;img src="44" width=60 height=60 offset=-7/&gt; được tính, tất cả &lt;img src="44" width=60 height=60 offset=-7/&gt; đã được tính trước đó sẽ biến thành &lt;img src="45" width=60 height=60 offset=-7/&gt;._x000d_
-_x000d_
-Các lượt quay còn lại chỉ được thực hiện nếu vẫn còn vị trí không chứa &lt;img src="45" width=60 height=60 offset=-7/&gt; lẫn &lt;img src="44" width=60 height=60 offset=-7/&gt;. Nếu tất cả_x000d_
-các vị trí đều được giữ lại, giá trị hiển thị trên đồng hồ jackpot GRAND sẽ được trao._x000d_
-_x000d_
-Một bộ reel khác được sử dụng trong Matsuri Feature. Tất cả các biểu tượng xuất hiện trên reel_x000d_
-ngoại trừ &lt;img src="45" width=60 height=60 offset=-7/&gt; và &lt;img src="44" width=60 height=60 offset=-7/&gt; sẽ bị làm mờ xám và không được tính. Việc phân bổ giải thưởng thay đổi_x000d_
+        <v xml:space="preserve">&lt;img src="44" width=60 height=60 offset=-7/&gt; được tính khi rơi trên màn hình. Nếu nhiều &lt;img src="44" width=60 height=60 offset=-7/&gt; cùng rơi trên màn hình, chúng sẽ được tính
+lần lượt từng cái một. Trước khi một &lt;img src="44" width=60 height=60 offset=-7/&gt; được tính, tất cả &lt;img src="44" width=60 height=60 offset=-7/&gt; đã được tính trước đó sẽ biến thành &lt;img src="45" width=60 height=60 offset=-7/&gt;.
+Các lượt quay còn lại chỉ được thực hiện nếu vẫn còn vị trí không chứa &lt;img src="45" width=60 height=60 offset=-7/&gt; lẫn &lt;img src="44" width=60 height=60 offset=-7/&gt;. Nếu tất cả
+các vị trí đều được giữ lại, giá trị hiển thị trên đồng hồ jackpot GRAND sẽ được trao.
+Một bộ reel khác được sử dụng trong Matsuri Feature. Tất cả các biểu tượng xuất hiện trên reel
+ngoại trừ &lt;img src="45" width=60 height=60 offset=-7/&gt; và &lt;img src="44" width=60 height=60 offset=-7/&gt; sẽ bị làm mờ xám và không được tính. Việc phân bổ giải thưởng thay đổi
 theo mức cược. Các giải thưởng tín dụng xuất hiện trên màn hình được trao đúng như hiển thị.</v>
       </c>
     </row>
@@ -3642,63 +3541,63 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C73" t="str" xml:space="preserve">
-        <v xml:space="preserve">During the base reel game, the Red Mystery Envelope Bonus may be Triggered at random._x000d_
-You will be shown a cash prize on top of the red envelope._x000d_
-The win from this bonus is x 50 based on the current bet value._x000d_
+        <v xml:space="preserve">During the base reel game, the Red Mystery Envelope Bonus may be Triggered at random.
+You will be shown a cash prize on top of the red envelope.
+The win from this bonus is x 50 based on the current bet value.
 After the prize is awarded, the game will continue as normal</v>
       </c>
       <c r="D73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Base Game 진행 중 Red Mystery Envelope Bonus가 무작위로 발동될 수 있습니다._x000d_
-붉은 봉투에 표시된 보상을 획득하게 되며,_x000d_
-현재 Bet 기준 x50 배의 당첨금이 지급됩니다._x000d_
+        <v xml:space="preserve">Base Game 진행 중 Red Mystery Envelope Bonus가 무작위로 발동될 수 있습니다.
+붉은 봉투에 표시된 보상을 획득하게 되며,
+현재 Bet 기준 x50 배의 당첨금이 지급됩니다.
 보상 지급 후 게임은 정상적으로 이어집니다.</v>
       </c>
       <c r="E73" t="str" xml:space="preserve">
-        <v xml:space="preserve">在基础卷轴游戏期间，可能会随机触发 Red Mystery Envelope Bonus。_x000d_
-红包上方将显示一份现金奖励。_x000d_
-此奖励的赢额为当前投注额的 x 50。_x000d_
+        <v xml:space="preserve">在基础卷轴游戏期间，可能会随机触发 Red Mystery Envelope Bonus。
+红包上方将显示一份现金奖励。
+此奖励的赢额为当前投注额的 x 50。
 奖励授予后，游戏将照常继续。</v>
       </c>
       <c r="F73" t="str" xml:space="preserve">
-        <v xml:space="preserve">在基礎捲軸遊戲期間，可能會隨機觸發 Red Mystery Envelope Bonus。_x000d_
-紅包上方將顯示一份現金獎勵。_x000d_
-此獎勵的贏額為當前投注額的 x 50。_x000d_
+        <v xml:space="preserve">在基礎捲軸遊戲期間，可能會隨機觸發 Red Mystery Envelope Bonus。
+紅包上方將顯示一份現金獎勵。
+此獎勵的贏額為當前投注額的 x 50。
 獎勵授予後，遊戲將照常繼續。</v>
       </c>
       <c r="G73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Sa panahon ng base reel game, maaaring ma-trigger nang random ang Red Mystery Envelope Bonus._x000d_
-Magpapakita sa iyo ng cash prize sa ibabaw ng red envelope._x000d_
-Ang panalo mula sa bonus na ito ay x 50 batay sa kasalukuyang bet value._x000d_
+        <v xml:space="preserve">Sa panahon ng base reel game, maaaring ma-trigger nang random ang Red Mystery Envelope Bonus.
+Magpapakita sa iyo ng cash prize sa ibabaw ng red envelope.
+Ang panalo mula sa bonus na ito ay x 50 batay sa kasalukuyang bet value.
 Pagkatapos igawad ang premyo, magpapatuloy ang laro gaya ng dati.</v>
       </c>
       <c r="H73" t="str" xml:space="preserve">
-        <v xml:space="preserve">ベースリールゲーム中、Red Mystery Envelope Bonus がランダムに発動することがあります。_x000d_
-赤い封筒の上にキャッシュ賞金が表示されます。_x000d_
-このボーナスの当選額は、現在のベット額の x 50 です。_x000d_
+        <v xml:space="preserve">ベースリールゲーム中、Red Mystery Envelope Bonus がランダムに発動することがあります。
+赤い封筒の上にキャッシュ賞金が表示されます。
+このボーナスの当選額は、現在のベット額の x 50 です。
 賞金が付与された後、ゲームは通常どおり続行されます。</v>
       </c>
       <c r="I73" t="str" xml:space="preserve">
-        <v xml:space="preserve">ในระหว่างเกมรีลพื้นฐาน Red Mystery Envelope Bonus อาจถูกกระตุ้นแบบสุ่ม_x000d_
-คุณจะเห็นรางวัลเงินสดแสดงอยู่เหนือซองแดง_x000d_
-รางวัลจากโบนัสนี้คือ x 50 โดยอิงตามค่าเดิมพันปัจจุบัน_x000d_
+        <v xml:space="preserve">ในระหว่างเกมรีลพื้นฐาน Red Mystery Envelope Bonus อาจถูกกระตุ้นแบบสุ่ม
+คุณจะเห็นรางวัลเงินสดแสดงอยู่เหนือซองแดง
+รางวัลจากโบนัสนี้คือ x 50 โดยอิงตามค่าเดิมพันปัจจุบัน
 หลังจากได้รับรางวัลแล้ว เกมจะดำเนินต่อไปตามปกติ</v>
       </c>
       <c r="J73" t="str" xml:space="preserve">
-        <v xml:space="preserve">During the base reel game, the Red Mystery Envelope Bonus may be Triggered at random._x000d_
-You will be shown a cash prize on top of the red envelope._x000d_
-The win from this bonus is x 50 based on the current bet value._x000d_
+        <v xml:space="preserve">During the base reel game, the Red Mystery Envelope Bonus may be Triggered at random.
+You will be shown a cash prize on top of the red envelope.
+The win from this bonus is x 50 based on the current bet value.
 After the prize is awarded, the game will continue as normal</v>
       </c>
       <c r="K73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Semasa base reel game, Red Mystery Envelope Bonus mungkin dicetuskan secara rawak._x000d_
-Anda akan ditunjukkan hadiah tunai di atas sampul merah._x000d_
-Kemenangan daripada bonus ini adalah x 50 berdasarkan nilai pusta semasa._x000d_
+        <v xml:space="preserve">Semasa base reel game, Red Mystery Envelope Bonus mungkin dicetuskan secara rawak.
+Anda akan ditunjukkan hadiah tunai di atas sampul merah.
+Kemenangan daripada bonus ini adalah x 50 berdasarkan nilai pusta semasa.
 Selepas hadiah dianugerahkan, permainan akan diteruskan seperti biasa.</v>
       </c>
       <c r="L73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Trong base reel game, Red Mystery Envelope Bonus có thể được kích hoạt một cách ngẫu nhiên._x000d_
-Bạn sẽ thấy một giải thưởng tiền mặt hiện trên chiếc bao đỏ._x000d_
-Tiền thắng từ bonus này là x 50 dựa trên giá trị cược hiện tại._x000d_
+        <v xml:space="preserve">Trong base reel game, Red Mystery Envelope Bonus có thể được kích hoạt một cách ngẫu nhiên.
+Bạn sẽ thấy một giải thưởng tiền mặt hiện trên chiếc bao đỏ.
+Tiền thắng từ bonus này là x 50 dựa trên giá trị cược hiện tại.
 Sau khi giải thưởng được trao, trò chơi sẽ tiếp tục như bình thường.</v>
       </c>
     </row>
@@ -3748,85 +3647,85 @@
         <v>Game &amp; Pay Info</v>
       </c>
       <c r="C75" t="str" xml:space="preserve">
-        <v xml:space="preserve">All win amounts are multiplied by the base bet._x000d_
-All values are displayed as actual coin wins._x000d_
-When winning with multiple symbols simultaneously, all win amounts are added together and paid as the total win._x000d_
-Only highest win paid per winning combination._x000d_
-In accordance with fair gaming practices, the outcome of each and every game is completely independent._x000d_
+        <v xml:space="preserve">All win amounts are multiplied by the base bet.
+All values are displayed as actual coin wins.
+When winning with multiple symbols simultaneously, all win amounts are added together and paid as the total win.
+Only highest win paid per winning combination.
+In accordance with fair gaming practices, the outcome of each and every game is completely independent.
 The chances of getting a particular outcome are always the same at the start of every game.</v>
       </c>
       <c r="D75" t="str" xml:space="preserve">
-        <v xml:space="preserve">모든 당첨금은 Base Bet을 기준으로 계산됩니다._x000d_
-표시되는 모든 수치는 실제 코인 당첨금입니다._x000d_
-여러 심볼 조합이 동시에 당첨된 경우,_x000d_
-각 당첨금은 합산되어 총 당첨금으로 지급됩니다._x000d_
-동일한 당첨 조합에서는 가장 높은 당첨금만 지급됩니다._x000d_
-공정한 게임 운영 원칙에 따라,_x000d_
-각 게임의 결과는 모두 독립적으로 결정됩니다._x000d_
+        <v xml:space="preserve">모든 당첨금은 Base Bet을 기준으로 계산됩니다.
+표시되는 모든 수치는 실제 코인 당첨금입니다.
+여러 심볼 조합이 동시에 당첨된 경우,
+각 당첨금은 합산되어 총 당첨금으로 지급됩니다.
+동일한 당첨 조합에서는 가장 높은 당첨금만 지급됩니다.
+공정한 게임 운영 원칙에 따라,
+각 게임의 결과는 모두 독립적으로 결정됩니다.
 특정 결과가 발생할 확률은 모든 게임 시작 시 항상 동일합니다.</v>
       </c>
       <c r="E75" t="str" xml:space="preserve">
-        <v xml:space="preserve">所有赢额均以基础投注额相乘计算。_x000d_
-所有数值均以实际金币赢额显示。_x000d_
-当同时以多个符号获胜时，所有赢额将相加并作为总赢额支付。_x000d_
-每个获胜组合仅支付最高赢额。_x000d_
-根据公平游戏原则，每一局游戏的结果都是完全独立的。_x000d_
+        <v xml:space="preserve">所有赢额均以基础投注额相乘计算。
+所有数值均以实际金币赢额显示。
+当同时以多个符号获胜时，所有赢额将相加并作为总赢额支付。
+每个获胜组合仅支付最高赢额。
+根据公平游戏原则，每一局游戏的结果都是完全独立的。
 在每局游戏开始时，获得某一特定结果的概率始终相同。</v>
       </c>
       <c r="F75" t="str" xml:space="preserve">
-        <v xml:space="preserve">所有贏額均以基礎投注額相乘計算。_x000d_
-所有數值均以實際金幣贏額顯示。_x000d_
-當同時以多個符號獲勝時，所有贏額將相加並作為總贏額支付。_x000d_
-每個獲勝組合僅支付最高贏額。_x000d_
-根據公平遊戲原則，每一局遊戲的結果都是完全獨立的。_x000d_
+        <v xml:space="preserve">所有贏額均以基礎投注額相乘計算。
+所有數值均以實際金幣贏額顯示。
+當同時以多個符號獲勝時，所有贏額將相加並作為總贏額支付。
+每個獲勝組合僅支付最高贏額。
+根據公平遊戲原則，每一局遊戲的結果都是完全獨立的。
 在每局遊戲開始時，獲得某一特定結果的概率始終相同。</v>
       </c>
       <c r="G75" t="str" xml:space="preserve">
-        <v xml:space="preserve">Lahat ng win amount ay minu-multiply sa base bet._x000d_
-Lahat ng halaga ay ipinapakita bilang aktwal na coin wins._x000d_
-Kapag nanalo gamit ang maraming simbolo nang sabay-sabay, lahat ng win amount ay pinagsasama-sama at binabayaran bilang total win._x000d_
-Ang pinakamataas na panalo lamang ang binabayaran sa bawat winning combination._x000d_
-Alinsunod sa fair gaming practices, ang resulta ng bawat laro ay ganap na independiyente._x000d_
+        <v xml:space="preserve">Lahat ng win amount ay minu-multiply sa base bet.
+Lahat ng halaga ay ipinapakita bilang aktwal na coin wins.
+Kapag nanalo gamit ang maraming simbolo nang sabay-sabay, lahat ng win amount ay pinagsasama-sama at binabayaran bilang total win.
+Ang pinakamataas na panalo lamang ang binabayaran sa bawat winning combination.
+Alinsunod sa fair gaming practices, ang resulta ng bawat laro ay ganap na independiyente.
 Ang tsansa na makakuha ng isang partikular na resulta ay palaging pareho sa simula ng bawat laro.</v>
       </c>
       <c r="H75" t="str" xml:space="preserve">
-        <v xml:space="preserve">すべての当選額はベースベットを乗じて計算されます。_x000d_
-すべての数値は実際のコイン獲得額として表示されます。_x000d_
-複数のシンボルで同時に当選した場合、すべての当選額が合算され、合計当選額として支払われます。_x000d_
-各当選組み合わせにつき、最高額の当選のみが支払われます。_x000d_
-公正なゲーム運営の原則に従い、各ゲームの結果は完全に独立しています。_x000d_
+        <v xml:space="preserve">すべての当選額はベースベットを乗じて計算されます。
+すべての数値は実際のコイン獲得額として表示されます。
+複数のシンボルで同時に当選した場合、すべての当選額が合算され、合計当選額として支払われます。
+各当選組み合わせにつき、最高額の当選のみが支払われます。
+公正なゲーム運営の原則に従い、各ゲームの結果は完全に独立しています。
 特定の結果が出る確率は、毎回のゲーム開始時において常に同じです。</v>
       </c>
       <c r="I75" t="str" xml:space="preserve">
-        <v xml:space="preserve">จำนวนเงินรางวัลทั้งหมดจะถูกคูณด้วยเดิมพันพื้นฐาน (base bet)_x000d_
-ค่าทั้งหมดจะแสดงเป็นจำนวนเหรียญที่ชนะจริง_x000d_
-เมื่อชนะด้วยสัญลักษณ์หลายตัวพร้อมกัน จำนวนเงินรางวัลทั้งหมดจะถูกนำมารวมกันและจ่ายเป็นรางวัลรวม_x000d_
-จ่ายเฉพาะรางวัลสูงสุดต่อหนึ่งชุดการชนะเท่านั้น_x000d_
-ตามหลักปฏิบัติของการเล่นเกมที่เป็นธรรม ผลลัพธ์ของแต่ละเกมเป็นอิสระจากกันโดยสมบูรณ์_x000d_
+        <v xml:space="preserve">จำนวนเงินรางวัลทั้งหมดจะถูกคูณด้วยเดิมพันพื้นฐาน (base bet)
+ค่าทั้งหมดจะแสดงเป็นจำนวนเหรียญที่ชนะจริง
+เมื่อชนะด้วยสัญลักษณ์หลายตัวพร้อมกัน จำนวนเงินรางวัลทั้งหมดจะถูกนำมารวมกันและจ่ายเป็นรางวัลรวม
+จ่ายเฉพาะรางวัลสูงสุดต่อหนึ่งชุดการชนะเท่านั้น
+ตามหลักปฏิบัติของการเล่นเกมที่เป็นธรรม ผลลัพธ์ของแต่ละเกมเป็นอิสระจากกันโดยสมบูรณ์
 โอกาสในการได้รับผลลัพธ์ใดผลลัพธ์หนึ่งจะเท่ากันเสมอเมื่อเริ่มต้นเกมแต่ละครั้ง</v>
       </c>
       <c r="J75" t="str" xml:space="preserve">
-        <v xml:space="preserve">All win amounts are multiplied by the base bet._x000d_
-All values are displayed as actual coin wins._x000d_
-When winning with multiple symbols simultaneously, all win amounts are added together and paid as the total win._x000d_
-Only highest win paid per winning combination._x000d_
-In accordance with fair gaming practices, the outcome of each and every game is completely independent._x000d_
+        <v xml:space="preserve">All win amounts are multiplied by the base bet.
+All values are displayed as actual coin wins.
+When winning with multiple symbols simultaneously, all win amounts are added together and paid as the total win.
+Only highest win paid per winning combination.
+In accordance with fair gaming practices, the outcome of each and every game is completely independent.
 The chances of getting a particular outcome are always the same at the start of every game.</v>
       </c>
       <c r="K75" t="str" xml:space="preserve">
-        <v xml:space="preserve">Semua jumlah kemenangan digandakan dengan base bet._x000d_
-Semua nilai dipaparkan sebagai kemenangan koin sebenar._x000d_
-Apabila menang dengan beberapa simbol secara serentak, semua jumlah kemenangan akan dicampur dan dibayar sebagai jumlah kemenangan keseluruhan._x000d_
-Hanya kemenangan tertinggi dibayar bagi setiap kombinasi kemenangan._x000d_
-Selaras dengan amalan permainan yang adil, keputusan setiap permainan adalah bebas sepenuhnya._x000d_
+        <v xml:space="preserve">Semua jumlah kemenangan digandakan dengan base bet.
+Semua nilai dipaparkan sebagai kemenangan koin sebenar.
+Apabila menang dengan beberapa simbol secara serentak, semua jumlah kemenangan akan dicampur dan dibayar sebagai jumlah kemenangan keseluruhan.
+Hanya kemenangan tertinggi dibayar bagi setiap kombinasi kemenangan.
+Selaras dengan amalan permainan yang adil, keputusan setiap permainan adalah bebas sepenuhnya.
 Peluang untuk mendapat keputusan tertentu adalah sama pada permulaan setiap permainan.</v>
       </c>
       <c r="L75" t="str" xml:space="preserve">
-        <v xml:space="preserve">Mọi khoản tiền thắng đều được nhân với base bet._x000d_
-Mọi giá trị được hiển thị theo số xu thắng thực tế._x000d_
-Khi thắng với nhiều biểu tượng cùng lúc, tất cả các khoản tiền thắng sẽ được cộng lại và chi trả như tổng tiền thắng._x000d_
-Chỉ khoản thắng cao nhất được chi trả cho mỗi tổ hợp thắng._x000d_
-Theo nguyên tắc chơi công bằng, kết quả của mỗi và từng ván chơi là hoàn toàn độc lập._x000d_
+        <v xml:space="preserve">Mọi khoản tiền thắng đều được nhân với base bet.
+Mọi giá trị được hiển thị theo số xu thắng thực tế.
+Khi thắng với nhiều biểu tượng cùng lúc, tất cả các khoản tiền thắng sẽ được cộng lại và chi trả như tổng tiền thắng.
+Chỉ khoản thắng cao nhất được chi trả cho mỗi tổ hợp thắng.
+Theo nguyên tắc chơi công bằng, kết quả của mỗi và từng ván chơi là hoàn toàn độc lập.
 Xác suất nhận được một kết quả cụ thể luôn giống nhau vào đầu mỗi ván chơi.</v>
       </c>
     </row>
@@ -3838,63 +3737,63 @@
         <v>Ingame Pop-up</v>
       </c>
       <c r="C76" t="str" xml:space="preserve">
-        <v xml:space="preserve">TOUCH A COIN TO REVEAL MATSURI SYMBOL OR &lt;img src = '86' height=60 offset=-12 /&gt;. _x000d_
-MATCH 3 MATSURI SYMBOLS TO AWARD A JACKPOT OR BONUS. REVEAL 3 &lt;img src = '86' height=60 offset=-12 /&gt;_x000d_
-TO UPGRADE THE JACKPOT OR BONUS AWARDED BY ONE LEVEL EXCEPT_x000d_
+        <v xml:space="preserve">TOUCH A COIN TO REVEAL MATSURI SYMBOL OR &lt;img src = '86' height=50 offset=-5 /&gt;. 
+MATCH 3 MATSURI SYMBOLS TO AWARD A JACKPOT OR BONUS. REVEAL 3 &lt;img src = '86' height=50 offset=-5 /&gt;
+TO UPGRADE THE JACKPOT OR BONUS AWARDED BY ONE LEVEL EXCEPT
 THE GRAND JACKPOT WHICH WILL BE AWARDED TWICE.</v>
       </c>
       <c r="D76" t="str" xml:space="preserve">
-        <v xml:space="preserve">코인을 터치해 마츠리 심볼 또는 &lt;img src = '86' height=60 offset=-12 /&gt;을 확인하세요._x000d_
-마츠리 심볼 3개 매치 시 잭팟 또는 보너스를 획득합니다. &lt;img src = '86' height=60 offset=-12 /&gt; 3개를 공개하면_x000d_
+        <v xml:space="preserve">코인을 터치해 마츠리 심볼 또는 &lt;img src = '86' height=50 offset=-5 /&gt;을 확인하세요.
+마츠리 심볼 3개 매치 시 잭팟 또는 보너스를 획득합니다. &lt;img src = '86' height=50 offset=-5 /&gt; 3개를 공개하면
 획득한 잭팟·보너스가 한 단계 업그레이드되며, 그랜드 잭팟의 경우 두 배로 지급됩니다.</v>
       </c>
       <c r="E76" t="str" xml:space="preserve">
-        <v xml:space="preserve">点击金币以揭示 Matsuri 符号或 &lt;img src = '86' height=60 offset=-12 /&gt;。_x000d_
-集齐 3 个 Matsuri 符号即可获得 JACKPOT 或 BONUS。揭示 3 个 &lt;img src = '86' height=60 offset=-12 /&gt;_x000d_
-可将所获得的 JACKPOT 或 BONUS 升级一个等级，但 GRAND JACKPOT_x000d_
+        <v xml:space="preserve">点击金币以揭示 Matsuri 符号或 &lt;img src = '86' height=50 offset=-5 /&gt;。
+集齐 3 个 Matsuri 符号即可获得 JACKPOT 或 BONUS。揭示 3 个 &lt;img src = '86' height=50 offset=-5 /&gt;
+可将所获得的 JACKPOT 或 BONUS 升级一个等级，但 GRAND JACKPOT
 将改为加倍授予。</v>
       </c>
       <c r="F76" t="str" xml:space="preserve">
-        <v xml:space="preserve">點擊金幣以揭示 Matsuri 符號或 &lt;img src = '86' height=60 offset=-12 /&gt;。_x000d_
-集齊 3 個 Matsuri 符號即可獲得 JACKPOT 或 BONUS。揭示 3 個 &lt;img src = '86' height=60 offset=-12 /&gt;_x000d_
-可將所獲得的 JACKPOT 或 BONUS 升級一個等級，但 GRAND JACKPOT_x000d_
+        <v xml:space="preserve">點擊金幣以揭示 Matsuri 符號或 &lt;img src = '86' height=50 offset=-5 /&gt;。
+集齊 3 個 Matsuri 符號即可獲得 JACKPOT 或 BONUS。揭示 3 個 &lt;img src = '86' height=50 offset=-5 /&gt;
+可將所獲得的 JACKPOT 或 BONUS 升級一個等級，但 GRAND JACKPOT
 將改為加倍授予。</v>
       </c>
       <c r="G76" t="str" xml:space="preserve">
-        <v xml:space="preserve">PINDUTIN ANG COIN PARA IPAKITA ANG MATSURI SYMBOL O &lt;img src = '86' height=60 offset=-12 /&gt;._x000d_
-ITUGMA ANG 3 MATSURI SYMBOL PARA MAKAKUHA NG JACKPOT O BONUS. KUNG MAIPAPAKITA ANG 3 &lt;img src = '86' height=60 offset=-12 /&gt;,_x000d_
-MAA-UPGRADE NG ISANG ANTAS ANG NAKUHANG JACKPOT O BONUS, MALIBAN SA_x000d_
-GRAND JACKPOT NA IGAGAWAD NANG DALAWANG BESES.</v>
+        <v xml:space="preserve">PINDUTIN ANG COIN PARA IPAKITA MATSURI SYMBOL O &lt;img src = '86' height=50 offset=-5 /&gt;.
+ITUGMA ANG 3 MATSURI SYMBOL PARA JACKPOT O BONUS.
+3 &lt;img src = '86' height=50 offset=-5 /&gt; NAG-A-UPGRADE NG GANTIMPALA NG 1 ANTAS.
+GRAND JACKPOT AAWARD NG DALAWANG BESES.</v>
       </c>
       <c r="H76" t="str" xml:space="preserve">
-        <v xml:space="preserve">コインをタッチして祭りシンボルまたは&lt;img src = '86' height=60 offset=-12 /&gt;を公開しよう。_x000d_
-祭りシンボルが3つ揃うとジャックポットまたはボーナスを獲得。&lt;img src = '86' height=60 offset=-12 /&gt;を_x000d_
-3つ公開すると、獲得したジャックポットまたはボーナスが1段階アップグレードされます。_x000d_
+        <v xml:space="preserve">コインをタッチして祭りシンボルまたは&lt;img src = '86' height=50 offset=-5 /&gt;を公開しよう。
+祭りシンボルが3つ揃うとジャックポットまたはボーナスを獲得。&lt;img src = '86' height=50 offset=-5 /&gt;を
+3つ公開すると、獲得したジャックポットまたはボーナスが1段階アップグレードされます。
 ただしグランドジャックポットの場合は2倍で付与されます。</v>
       </c>
       <c r="I76" t="str" xml:space="preserve">
-        <v xml:space="preserve">แตะเหรียญเพื่อเปิดเผยสัญลักษณ์ MATSURI หรือ &lt;img src = '86' height=60 offset=-12 /&gt;_x000d_
-จับคู่สัญลักษณ์ MATSURI ครบ 3 ตัวเพื่อรับ JACKPOT หรือ BONUS_x000d_
-หากเปิดเผย &lt;img src = '86' height=60 offset=-12 /&gt; ครบ 3 ตัว รางวัล JACKPOT หรือ BONUS ที่ได้รับจะถูกอัปเกรดขึ้นหนึ่งระดับ_x000d_
+        <v xml:space="preserve">แตะเหรียญเพื่อเปิดเผยสัญลักษณ์ MATSURI หรือ &lt;img src = '86' height=50 offset=-5 /&gt;
+จับคู่สัญลักษณ์ MATSURI ครบ 3 ตัวเพื่อรับ JACKPOT หรือ BONUS
+หากเปิดเผย &lt;img src = '86' height=50 offset=-5 /&gt; ครบ 3 ตัว รางวัล JACKPOT หรือ BONUS ที่ได้รับจะถูกอัปเกรดขึ้นหนึ่งระดับ
 ยกเว้น GRAND JACKPOT ซึ่งจะมอบรางวัลให้สองเท่า</v>
       </c>
       <c r="J76" t="str" xml:space="preserve">
-        <v xml:space="preserve">TOUCH A COIN TO REVEAL MATSURI SYMBOL OR &lt;img src = '86' height=60 offset=-12 /&gt;. _x000d_
-MATCH 3 MATSURI SYMBOLS TO AWARD A JACKPOT OR BONUS. REVEAL 3 &lt;img src = '86' height=60 offset=-12 /&gt;_x000d_
-TO UPGRADE THE JACKPOT OR BONUS AWARDED BY ONE LEVEL EXCEPT_x000d_
+        <v xml:space="preserve">TOUCH A COIN TO REVEAL MATSURI SYMBOL OR &lt;img src = '86' height=50 offset=-5 /&gt;. 
+MATCH 3 MATSURI SYMBOLS TO AWARD A JACKPOT OR BONUS. REVEAL 3 &lt;img src = '86' height=50 offset=-5 /&gt;
+TO UPGRADE THE JACKPOT OR BONUS AWARDED BY ONE LEVEL EXCEPT
 THE GRAND JACKPOT WHICH WILL BE AWARDED TWICE.</v>
       </c>
       <c r="K76" t="str" xml:space="preserve">
-        <v xml:space="preserve">SENTUH KOIN UNTUK MENDEDAHKAN MATSURI SYMBOL ATAU &lt;img src = '86' height=60 offset=-12 /&gt;._x000d_
-PADANKAN 3 MATSURI SYMBOL UNTUK MENDAPAT JACKPOT ATAU BONUS. DEDAHKAN 3 &lt;img src = '86' height=60 offset=-12 /&gt;_x000d_
-UNTUK MENAIK TARAF JACKPOT ATAU BONUS YANG DIANUGERAHKAN SEBANYAK SATU TAHAP,_x000d_
-KECUALI GRAND JACKPOT YANG AKAN DIANUGERAHKAN DUA KALI.</v>
+        <v xml:space="preserve">SENTUH KOIN UNTUK BUKA MATSURI SYMBOL ATAU &lt;img src = '86' height=36 offset=-8 /&gt;.
+PADANKAN 3 MATSURI SYMBOL UNTUK JACKPOT/BONUS.
+3 &lt;img src = '86' height=36 offset=-8 /&gt; NAIK TARAF GANJARAN 1 TAHAP.
+GRAND JACKPOT DIANUGERAH DUA KALI.</v>
       </c>
       <c r="L76" t="str" xml:space="preserve">
-        <v xml:space="preserve">CHẠM VÀO ĐỒNG XU ĐỂ MỞ MATSURI SYMBOL HOẶC &lt;img src = '86' height=60 offset=-12 /&gt;._x000d_
-GHÉP 3 MATSURI SYMBOL ĐỂ NHẬN JACKPOT HOẶC BONUS. MỞ ĐƯỢC 3 &lt;img src = '86' height=60 offset=-12 /&gt;_x000d_
-SẼ NÂNG JACKPOT HOẶC BONUS ĐÃ TRAO LÊN MỘT CẤP,_x000d_
-NGOẠI TRỪ GRAND JACKPOT SẼ ĐƯỢC TRAO GẤP ĐÔI.</v>
+        <v xml:space="preserve">CHẠM ĐỒNG XU ĐỂ MỞ MATSURI SYMBOL HOẶC &lt;img src = '86' height=50 offset=-5 /&gt;.
+GHÉP 3 MATSURI SYMBOL ĐỂ NHẬN JACKPOT/BONUS.
+MỞ ĐƯỢC 3 &lt;img src = '86' height=50 offset=-5 /&gt;SẼ NÂNG THƯỞNG 1 CẤP.
+GRAND JACKPOT SẼ TRAO THƯỞNG GẤP ĐÔI.</v>
       </c>
     </row>
     <row r="77">

</xml_diff>

<commit_message>
Fix notion bugs (v4) + Update sounds
</commit_message>
<xml_diff>
--- a/LocalizationStringTable.xlsx
+++ b/LocalizationStringTable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CocosProject\CarnivalNeko\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{874C4524-D63C-44FE-82BF-184B7D4A67AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FB6E7C-E725-48D7-9B1E-3267D1DDF74D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1609,79 +1609,6 @@
     <t>UI_POPUP_PAY_PAGE3_CONTENTS1</t>
   </si>
   <si>
-    <t xml:space="preserve">
-Each Trail Symbol that lands during the base game will fly into corresponding colored fortune pouch.
-Any Trail Symbol may trigger the corresponding fortune pouch.
-More than one fortune pouch can be triggered on a single spin.
-If fortune pouch(s) are triggered, the corresponding feature will start.
-The Accumulation of Trail Symbols over time in the BLUE, RED and GREEN fortune pouches have no
-effect on triggering the JACKPOT FEATURE or MATSURI FEATURE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Base game에서 획득한 Trail Symbol은 해당 색상의 복주머니로 수집됩니다.
-Trail Symbol은 해당 복주머니 Feature를 발동할 수 있으며, 하나의 스핀에서 여러 개의 복주머니가 동시에 발동될 수 있습니다.
-복주머니가 발동되면 해당 Feature가 시작됩니다.
-파란색, 빨간색, 녹색 복주머니에 누적된 Trail Symbol은 JACKPOT FEATURE 또는 MATSURI FEATURE의 발동 확률에 영향을 주지 않습니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-主游戏期间每个落定的 Trail 符号都会飞入对应颜色的福袋。
-任意 Trail 符号都可触发其对应的福袋。
-单次旋转中可同时触发多个福袋。
-若福袋被触发，对应的功能将随之启动。
-Trail 符号在蓝色、红色和绿色福袋中长期累积，不会影响 JACKPOT FEATURE 或 MATSURI FEATURE 的触发。</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-主遊戲期間每個落定的 Trail 符號都會飛入對應顏色的福袋。
-任意 Trail 符號都可觸發其對應的福袋。
-單次旋轉中可同時觸發多個福袋。
-若福袋被觸發，對應的功能將隨之啟動。
-Trail 符號在藍色、紅色與綠色福袋中長期累積，不會影響 JACKPOT FEATURE 或 MATSURI FEATURE 的觸發。</t>
-  </si>
-  <si>
-    <t>Ang bawat Trail Symbol na lalapag sa base game ay lilipad papunta sa katugmang kulay na fortune pouch.
-Anumang Trail Symbol ay maaaring mag-trigger ng katugmang fortune pouch.
-Maaaring ma-trigger ang higit sa isang fortune pouch sa iisang spin.
-Kapag na-trigger ang (mga) fortune pouch, magsisimula ang katugmang feature.
-Ang pag-iipon ng mga Trail Symbol sa paglipas ng panahon sa BLUE, RED, at GREEN na fortune pouch ay walang epekto sa pag-trigger ng JACKPOT FEATURE o MATSURI FEATURE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-ベースゲーム中に着地した各 Trail シンボルは、対応する色の福袋へ飛び込みます。
-いずれの Trail シンボルでも、対応する福袋を発動させることがあります。
-1回のスピンで複数の福袋が発動することがあります。
-福袋が発動すると、対応するフィーチャーが開始します。
-青・赤・緑の福袋に Trail シンボルが時間とともに蓄積されても、JACKPOT FEATURE や MATSURI FEATURE の発動には影響しません。</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-สัญลักษณ์ Trail แต่ละตัวที่ตกลงมาในเกมหลักจะลอยเข้าสู่ถุงนำโชค (fortune pouch) ที่มีสีตรงกัน
-สัญลักษณ์ Trail ใด ๆ ก็สามารถกระตุ้นถุงนำโชคที่ตรงกันได้
-สามารถกระตุ้นถุงนำโชคได้มากกว่าหนึ่งใบในการหมุนเพียงครั้งเดียว
-เมื่อถุงนำโชคถูกกระตุ้น ฟีเจอร์ที่สอดคล้องกันจะเริ่มต้นขึ้น
-การสะสมสัญลักษณ์ Trail เมื่อเวลาผ่านไปในถุงนำโชคสีน้ำเงิน สีแดง และสีเขียว ไม่มีผลต่อการกระตุ้น JACKPOT FEATURE หรือ MATSURI FEATURE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Setiap Trail Symbol yang mendarat semasa base game akan terbang masuk ke dalam fortune pouch yang sewarna dengannya.
-Mana-mana Trail Symbol boleh mencetuskan fortune pouch yang sepadan.
-Lebih daripada satu fortune pouch boleh dicetuskan dalam satu spin.
-Jika fortune pouch dicetuskan, feature yang sepadan akan bermula.
-Pengumpulan Trail Symbol dari masa ke masa dalam fortune pouch BIRU, MERAH dan HIJAU tidak
-memberi kesan kepada pencetusan JACKPOT FEATURE atau MATSURI FEATURE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Mọi Trail Symbol xuất hiện trong base game sẽ bay vào túi phúc (fortune pouch) cùng màu tương ứng.
-Bất kỳ Trail Symbol nào cũng có thể kích hoạt túi phúc tương ứng.
-Có thể kích hoạt nhiều hơn một túi phúc trong cùng một lượt quay.
-Khi túi phúc được kích hoạt, feature tương ứng sẽ bắt đầu.
-Việc tích lũy Trail Symbol theo thời gian trong các túi phúc XANH DƯƠNG, ĐỎ và XANH LÁ không
-ảnh hưởng đến việc kích hoạt JACKPOT FEATURE hay MATSURI FEATURE.</t>
-  </si>
-  <si>
     <t>UI_POPUP_PAY_PAGE4_TITLE1</t>
   </si>
   <si>
@@ -1701,36 +1628,6 @@
   </si>
   <si>
     <t>UI_POPUP_PAY_PAGE4_CONTENTS1</t>
-  </si>
-  <si>
-    <t>Any Red Trail Symbol landing in the Red fortune pouch. May trigger the
-JACKPOT FEATURE</t>
-  </si>
-  <si>
-    <t>빨간 복주머니에 수집된 Red Trail Symbol은 JACKPOT FEATURE를 발동 시킬 수 있습니다.</t>
-  </si>
-  <si>
-    <t>任意落入红色福袋的红色 Trail 符号，均有机会触发 JACKPOT FEATURE。</t>
-  </si>
-  <si>
-    <t>任意落入紅色福袋的紅色 Trail 符號，皆有機會觸發 JACKPOT FEATURE。</t>
-  </si>
-  <si>
-    <t>Anumang Red Trail Symbol na lalapag sa Red na fortune pouch ay maaaring mag-trigger ng JACKPOT FEATURE.</t>
-  </si>
-  <si>
-    <t>赤色の福袋に着地したいずれの赤色 Trail シンボルも、JACKPOT FEATURE を発動させることがあります。</t>
-  </si>
-  <si>
-    <t>สัญลักษณ์ Red Trail ใด ๆ ที่ตกลงในถุงนำโชคสีแดง อาจกระตุ้น JACKPOT FEATURE ได้</t>
-  </si>
-  <si>
-    <t>Mana-mana Red Trail Symbol yang mendarat dalam fortune pouch Merah boleh mencetuskan
-JACKPOT FEATURE</t>
-  </si>
-  <si>
-    <t>Bất kỳ Red Trail Symbol nào rơi vào túi phúc Đỏ đều có thể kích hoạt
-JACKPOT FEATURE</t>
   </si>
   <si>
     <t>UI_POPUP_PAY_PAGE4_CONTENTS2</t>
@@ -1838,46 +1735,7 @@
     <t>UI_POPUP_PAY_PAGE5_TITLE1</t>
   </si>
   <si>
-    <t>COLLECTION FORTUNE POUCH</t>
-  </si>
-  <si>
-    <t>收集福袋</t>
-  </si>
-  <si>
-    <t>コレクション福袋</t>
-  </si>
-  <si>
-    <t>ถุงนำโชคสะสม</t>
-  </si>
-  <si>
     <t>UI_POPUP_PAY_PAGE5_CONTENTS1</t>
-  </si>
-  <si>
-    <t>FORTUNE POUCHS TRIGGERED FEATURE AWARDED GRID STARTER SYMBOLS</t>
-  </si>
-  <si>
-    <t>복주머니 발동 FEATURE 보상 GRID 시작 SYMBOLS</t>
-  </si>
-  <si>
-    <t>已触发的福袋 获得的功能 网格 初始符号</t>
-  </si>
-  <si>
-    <t>已觸發的福袋 獲得的功能 網格 起始符號</t>
-  </si>
-  <si>
-    <t>FORTUNE POUCHS TRIGGERED NA-AWARD NA FEATURE GRID STARTER SYMBOLS</t>
-  </si>
-  <si>
-    <t>発動した福袋 付与されるフィーチャー グリッド 初期シンボル</t>
-  </si>
-  <si>
-    <t>ถุงนำโชคที่ถูกกระตุ้น ฟีเจอร์ที่ได้รับ กริด สัญลักษณ์เริ่มต้น</t>
-  </si>
-  <si>
-    <t>FORTUNE POUCH DICETUSKAN FEATURE DIANUGERAHKAN GRID SIMBOL PERMULAAN</t>
-  </si>
-  <si>
-    <t>TÚI PHÚC ĐƯỢC KÍCH HOẠT FEATURE ĐƯỢC TRAO GRID BIỂU TƯỢNG KHỞI ĐẦU</t>
   </si>
   <si>
     <t>UI_POPUP_PAY_PAGE6_TITLE1</t>
@@ -2404,71 +2262,187 @@
     <t>Bất kỳ {count} &lt;img src = '45' height=60 offset=-11 /&gt;và &lt;img src = '44' height=60 offset=-11 /&gt; trao Grand Jackpot</t>
   </si>
   <si>
-    <t>코인을 터치해 마츠리 심볼 또는 &lt;img src = '86' height=45 offset = -5 /&gt;.을 확인하세요.
-마츠리 심볼 3개 매치 시 잭팟 또는 보너스를 획득합니다.
-&lt;img src = '86' height=45 offset = -5 /&gt;. 3개를 공개하면 잭팟·보너스가 1단계 업그레이드됩니다.
-그랜드 잭팟은 두 배로 지급됩니다.</t>
-  </si>
-  <si>
-    <t>แตะเหรียญเพื่อเปิดสัญลักษณ์ MATSURI หรือ &lt;img src = '86' height=45 offset = -5 /&gt;.
-จับคู่ MATSURI ครบ 3 ตัวเพื่อรับ JACKPOT หรือ BONUS
-เปิด &lt;img src = '86' height=45 offset = -5 /&gt;. ครบ 3 ตัว รางวัลจะอัปเกรดขึ้น 1 ระดับ
-GRAND JACKPOT จะมอบรางวัลสองเท่า</t>
-  </si>
-  <si>
-    <t>TOUCH A COIN TO REVEAL MATSURI SYMBOL OR &lt;img src = '86' height=45 offset = -5 /&gt;.
-MATCH 3 MATSURI SYMBOLS FOR JACKPOT/BONUS.
-REVEAL 3 &lt;img src = '86' height=45 offset = -5 /&gt;. TO UPGRADE THE PRIZE 1 LEVEL.
-GRAND JACKPOT IS AWARDED TWICE.</t>
-  </si>
-  <si>
-    <t>点击金币以揭示 Matsuri 符号或 &lt;img src = '86' height=45 offset = -5 /&gt;.
-集齐 3 个 Matsuri 符号即可获得 JACKPOT 或 BONUS。
-揭示 3 个 &lt;img src = '86' height=45 offset = -5 /&gt;. 可将奖励升级一个等级。
-GRAND JACKPOT 将加倍授予。</t>
-  </si>
-  <si>
-    <t>點擊金幣以揭示 Matsuri 符號或 &lt;img src = '86' height=45 offset = -5 /&gt;.
-集齊 3 個 Matsuri 符號即可獲得 JACKPOT 或 BONUS。
-揭示 3 個 &lt;img src = '86' height=45 offset = -5 /&gt;. 可將獎勵升級一個等級。
-GRAND JACKPOT 將加倍授予。</t>
-  </si>
-  <si>
-    <t>PINDUTIN ANG COIN PARA IPAKITA MATSURI O &lt;img src = '86' height=45 offset = -5 /&gt;.
-ITUGMA ANG 3 MATSURI PARA JACKPOT O BONUS.
-3 &lt;img src = '86' height=45 offset = -5 /&gt;. UPGRADE NG GANTIMPALA NG 1 ANTAS.
-GRAND JACKPOT IGAWAD NG DALAWANG BESES.</t>
-  </si>
-  <si>
-    <t>コインをタッチして祭りシンボルまたは&lt;img src = '86' height=45 offset = -5 /&gt;.を公開
-祭りシンボル3つでジャックポットまたはボーナス獲得。
-&lt;img src = '86' height=45 offset = -5 /&gt;.を3つ公開すると賞が1段階アップグレード。
-グランドジャックポットは2倍で付与。</t>
-  </si>
-  <si>
-    <t>SENTUH KOIN UNTUK BUKA MATSURI SYMBOL ATAU &lt;img src = '86' height=45 offset = -5 /&gt;.
-PADANKAN 3 MATSURI SYMBOL UNTUK JACKPOT/BONUS.
-3 &lt;img src = '86' height=45 offset = -5 /&gt;. NAIK TARAF GANJARAN 1 TAHAP.
-GRAND JACKPOT DIANUGERAH DUA KALI.</t>
-  </si>
-  <si>
-    <t>CHẠM ĐỒNG XU ĐỂ MỞ MATSURI SYMBOL HOẶC &lt;img src = '86' height=45 offset = -5 /&gt;.
-GHÉP 3 MATSURI SYMBOL ĐỂ NHẬN JACKPOT/BONUS.
-MỞ ĐƯỢC 3 &lt;img src = '86' height=45 offset = -5 /&gt;. SẼ NÂNG THƯỞNG 1 CẤP.
-GRAND JACKPOT SẼ TRAO THƯỞNG GẤP ĐÔI.</t>
+    <t>TOUCH A COIN! MATCH 3 MATSURI SYMBOLS TO WIN A JACKPOT BONUS.
+REVEAL 3 UPGRADE SYMBOLS TO UPGRADE BY ONE LEVEL (GRAND JACKPOT PAYS DOUBLE).</t>
+  </si>
+  <si>
+    <t>코인을 터치! 마츠리 3개 매치 시 잭팟 보너스 획득, 업그레이드 심볼 3개 시 한 단계 상승(그랜드 잭팟은 2배).</t>
+  </si>
+  <si>
+    <t>点击金币！集齐3个祭典（Matsuri）符号即可赢得头奖或奖励。开出3个升级符号可将奖励提升一级（超级头奖翻倍派发）。</t>
+  </si>
+  <si>
+    <t>點擊金幣！集齊3個祭典（Matsuri）符號即可贏得頭獎或獎勵。開出3個升級符號可將獎勵提升一級（超級頭獎加倍派發）。</t>
+  </si>
+  <si>
+    <t>PINDUTIN ANG BARYA! TUMUGMA NG 3 MATSURI SYMBOL PARA MANALO NG JACKPOT BONUS. MAGBUNYAG NG 3 UPGRADE SYMBOL PARA UMANGAT NG ISANG ANTAS (DOBLE ANG BAYAD SA GRAND JACKPOT).</t>
+  </si>
+  <si>
+    <t>コインをタッチ！祭りシンボルを3つそろえるとジャックポットまたはボーナスを獲得。アップグレードシンボルを3つ出すと、獲得した賞が1段階アップ（グランドジャックポットは2倍で支払い）。</t>
+  </si>
+  <si>
+    <t>แตะเหรียญ! จับคู่สัญลักษณ์มัตสึริ (Matsuri) 3 ตัว เพื่อรับแจ็กพอตหรือโบนัส เปิดสัญลักษณ์อัปเกรด 3 ตัว เพื่อเลื่อนระดับขึ้นหนึ่งขั้น (แกรนด์แจ็กพอตจ่ายเป็นสองเท่า)</t>
+  </si>
+  <si>
+    <t>SENTUH SYILING! PADANKAN 3 SIMBOL MATSURI UNTUK MEMENANGI JACKPOT ATAU BONUS. DEDAHKAN 3 SIMBOL NAIK TARAF UNTUK NAIK SATU PERINGKAT (GRAND JACKPOT DIBAYAR DUA KALI GANDA).</t>
+  </si>
+  <si>
+    <t>CHẠM VÀO ĐỒNG XU! GHÉP 3 BIỂU TƯỢNG MATSURI ĐỂ THẮNG JACKPOT HOẶC TIỀN THƯỞNG. MỞ 3 BIỂU TƯỢNG NÂNG CẤP ĐỂ TĂNG MỘT CẤP (GRAND JACKPOT TRẢ GẤP ĐÔI).</t>
+  </si>
+  <si>
+    <t>Trail Symbols collected during the Base Game are gathered into the fortune Pot of the matching color.
+A Trail Symbol can trigger the Feature of its fortune Pot, and multiple Pots can be triggered on a single spin.
+When a Pot is triggered, the corresponding Feature starts.
+Trail Symbols accumulated in the BLUE, RED and GREEN fortune Pots do not affect the chance of triggering the JACKPOT FEATURE or MATSURI FEATURE.</t>
+  </si>
+  <si>
+    <t>Base game에서 획득한 Trail Symbol은 해당 색상의 단지로 수집됩니다.
+Trail Symbol은 해당 단지의 Feature를 발동할 수 있으며, 하나의 스핀에서 여러 개의 단지가 동시에 발동될 수 있습니다.
+단지가 발동되면 해당 Feature가 시작됩니다.
+파란색, 빨간색, 녹색 단지에 누적된 Trail Symbol은 JACKPOT FEATURE 또는 MATSURI FEATURE의 발동 확률에 영향을 주지 않습니다.</t>
+  </si>
+  <si>
+    <t>在Base Game中获得的Trail Symbol会被收集到对应颜色的福罐中。
+Trail Symbol可触发所属福罐的Feature，单次旋转中可同时触发多个福罐。
+福罐被触发后，对应的Feature随即开始。
+累积在蓝色、红色和绿色福罐中的Trail Symbol不会影响JACKPOT FEATURE或MATSURI FEATURE的触发概率。</t>
+  </si>
+  <si>
+    <t>在Base Game中獲得的Trail Symbol會被收集到對應顏色的福罐中。
+Trail Symbol可觸發所屬福罐的Feature，單次旋轉中可同時觸發多個福罐。
+福罐被觸發後，對應的Feature隨即開始。
+累積在藍色、紅色與綠色福罐中的Trail Symbol不會影響JACKPOT FEATURE或MATSURI FEATURE的觸發機率。</t>
+  </si>
+  <si>
+    <t>Ang mga Trail Symbol na nakuha sa Base Game ay naiipon sa fortune Pot na katugma ng kulay nito.
+Maaaring i-trigger ng Trail Symbol ang Feature ng fortune Pot na iyon, at maaaring ma-trigger ang maraming Pot sa isang spin.
+Kapag na-trigger ang Pot, magsisimula ang katugmang Feature.
+Ang mga Trail Symbol na naipon sa BLUE, RED at GREEN na fortune Pot ay hindi nakakaapekto sa tsansang ma-trigger ang JACKPOT FEATURE o MATSURI FEATURE.</t>
+  </si>
+  <si>
+    <t>ベースゲームで獲得したTrail Symbolは、対応する色の福壺に集められます。
+Trail Symbolはその福壺のFeatureを発動でき、1回のスピンで複数の福壺が同時に発動することがあります。
+福壺が発動すると、対応するFeatureが開始します。
+青・赤・緑の福壺に蓄積されたTrail Symbolは、JACKPOT FEATUREまたはMATSURI FEATUREの発動確率に影響しません。</t>
+  </si>
+  <si>
+    <t>สัญลักษณ์ Trail ที่ได้รับใน Base Game จะถูกเก็บรวบรวมไว้ในไหนำโชคที่มีสีตรงกัน
+สัญลักษณ์ Trail สามารถกระตุ้น Feature ของไหนำโชคนั้นได้ และในการหมุนเพียงครั้งเดียวอาจกระตุ้นไหนำโชคได้หลายใบพร้อมกัน
+เมื่อไหนำโชคถูกกระตุ้น Feature ที่สอดคล้องกันจะเริ่มต้นขึ้น
+สัญลักษณ์ Trail ที่สะสมอยู่ในไหนำโชคสีน้ำเงิน สีแดง และสีเขียว ไม่มีผลต่อโอกาสในการกระตุ้น JACKPOT FEATURE หรือ MATSURI FEATURE</t>
+  </si>
+  <si>
+    <t>Trail Symbol yang diperoleh semasa Base Game akan dikumpulkan ke dalam fortune Pot yang sewarna dengannya.
+Trail Symbol boleh mencetuskan Feature bagi fortune Pot tersebut, dan beberapa Pot boleh dicetuskan dalam satu spin.
+Apabila Pot dicetuskan, Feature yang sepadan akan bermula.
+Trail Symbol yang terkumpul dalam fortune Pot BIRU, MERAH dan HIJAU tidak mempengaruhi peluang pencetusan JACKPOT FEATURE atau MATSURI FEATURE.</t>
+  </si>
+  <si>
+    <t>Trail Symbol thu được trong Base Game sẽ được thu thập vào hũ phúc có màu tương ứng.
+Trail Symbol có thể kích hoạt Feature của hũ phúc đó, và nhiều hũ phúc có thể được kích hoạt cùng lúc trong một lượt quay.
+Khi hũ phúc được kích hoạt, Feature tương ứng sẽ bắt đầu.
+Trail Symbol tích lũy trong các hũ phúc XANH DƯƠNG, ĐỎ và XANH LÁ không ảnh hưởng đến xác suất kích hoạt JACKPOT FEATURE hay MATSURI FEATURE.</t>
+  </si>
+  <si>
+    <t>Any Red Trail Symbol landing in the Red fortune Pot. May trigger the
+JACKPOT FEATURE</t>
+  </si>
+  <si>
+    <t>빨간 단지에 수집된 Red Trail Symbol은 JACKPOT FEATURE를 발동 시킬 수 있습니다.</t>
+  </si>
+  <si>
+    <t>任意落入红色福罐的红色 Trail 符号，均有机会触发 JACKPOT FEATURE。</t>
+  </si>
+  <si>
+    <t>任意落入紅色福罐的紅色 Trail 符號，皆有機會觸發 JACKPOT FEATURE。</t>
+  </si>
+  <si>
+    <t>Anumang Red Trail Symbol na lalapag sa Red na fortune Pot ay maaaring mag-trigger ng JACKPOT FEATURE.</t>
+  </si>
+  <si>
+    <t>赤色の福壺に着地したいずれの赤色 Trail シンボルも、JACKPOT FEATURE を発動させることがあります。</t>
+  </si>
+  <si>
+    <t>สัญลักษณ์ Red Trail ใด ๆ ที่ตกลงในไหนำโชคสีแดง อาจกระตุ้น JACKPOT FEATURE ได้</t>
+  </si>
+  <si>
+    <t>Mana-mana Red Trail Symbol yang mendarat dalam fortune Pot Merah boleh mencetuskan
+JACKPOT FEATURE</t>
+  </si>
+  <si>
+    <t>Bất kỳ Red Trail Symbol nào rơi vào hũ phúc Đỏ đều có thể kích hoạt
+JACKPOT FEATURE</t>
+  </si>
+  <si>
+    <t>FORTUNE POTS TRIGGERED FEATURE AWARDED GRID STARTER SYMBOLS</t>
+  </si>
+  <si>
+    <t>단지 발동 FEATURE 보상 GRID 시작 SYMBOLS</t>
+  </si>
+  <si>
+    <t>已触发的福罐 获得的功能 网格 初始符号</t>
+  </si>
+  <si>
+    <t>已觸發的福罐 獲得的功能 網格 起始符號</t>
+  </si>
+  <si>
+    <t>FORTUNE POTS TRIGGERED NA-AWARD NA FEATURE GRID STARTER SYMBOLS</t>
+  </si>
+  <si>
+    <t>発動した福壺 付与されるフィーチャー グリッド 初期シンボル</t>
+  </si>
+  <si>
+    <t>ไหนำโชคที่ถูกกระตุ้น ฟีเจอร์ที่ได้รับ กริด สัญลักษณ์เริ่มต้น</t>
+  </si>
+  <si>
+    <t>FORTUNE POT DICETUSKAN FEATURE DIANUGERAHKAN GRID SIMBOL PERMULAAN</t>
+  </si>
+  <si>
+    <t>HŨ PHÚC ĐƯỢC KÍCH HOẠT FEATURE ĐƯỢC TRAO GRID BIỂU TƯỢNG KHỞI ĐẦU</t>
+  </si>
+  <si>
+    <t>COLLECTION FORTUNE POT</t>
+  </si>
+  <si>
+    <t>收集福罐</t>
+  </si>
+  <si>
+    <t>コレクション福壺</t>
+  </si>
+  <si>
+    <t>ไหนำโชคสะสม</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Malgun Gothic"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Malgun Gothic"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2479,7 +2453,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -2487,14 +2461,92 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2830,8 +2882,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L77"/>
+  <dimension ref="A1:Z77"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="112.125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -4657,7 +4712,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>445</v>
       </c>
@@ -4695,7 +4750,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>454</v>
       </c>
@@ -4733,7 +4788,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>464</v>
       </c>
@@ -4771,7 +4826,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>473</v>
       </c>
@@ -4809,7 +4864,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>483</v>
       </c>
@@ -4847,7 +4902,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>488</v>
       </c>
@@ -4885,7 +4940,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:26" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>498</v>
       </c>
@@ -4923,846 +4978,916 @@
         <v>499</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+    <row r="56" spans="1:26" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
         <v>504</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C56" s="4" t="s">
+        <v>635</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>636</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>637</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>638</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>639</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>640</v>
+      </c>
+      <c r="I56" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="J56" s="4" t="s">
+        <v>635</v>
+      </c>
+      <c r="K56" s="4" t="s">
+        <v>642</v>
+      </c>
+      <c r="L56" s="4" t="s">
+        <v>643</v>
+      </c>
+      <c r="M56" s="6"/>
+      <c r="N56" s="6"/>
+      <c r="O56" s="6"/>
+      <c r="P56" s="6"/>
+      <c r="Q56" s="6"/>
+      <c r="R56" s="6"/>
+      <c r="S56" s="6"/>
+      <c r="T56" s="6"/>
+      <c r="U56" s="6"/>
+      <c r="V56" s="6"/>
+      <c r="W56" s="6"/>
+      <c r="X56" s="6"/>
+      <c r="Y56" s="6"/>
+      <c r="Z56" s="6"/>
+    </row>
+    <row r="57" spans="1:26" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
         <v>505</v>
-      </c>
-      <c r="D56" t="s">
-        <v>506</v>
-      </c>
-      <c r="E56" t="s">
-        <v>507</v>
-      </c>
-      <c r="F56" t="s">
-        <v>508</v>
-      </c>
-      <c r="G56" t="s">
-        <v>509</v>
-      </c>
-      <c r="H56" t="s">
-        <v>510</v>
-      </c>
-      <c r="I56" t="s">
-        <v>511</v>
-      </c>
-      <c r="J56" t="s">
-        <v>505</v>
-      </c>
-      <c r="K56" t="s">
-        <v>512</v>
-      </c>
-      <c r="L56" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>514</v>
       </c>
       <c r="B57" t="s">
         <v>465</v>
       </c>
       <c r="C57" t="s">
-        <v>515</v>
+        <v>506</v>
       </c>
       <c r="D57" t="s">
-        <v>515</v>
+        <v>506</v>
       </c>
       <c r="E57" t="s">
-        <v>516</v>
+        <v>507</v>
       </c>
       <c r="F57" t="s">
-        <v>517</v>
+        <v>508</v>
       </c>
       <c r="G57" t="s">
-        <v>515</v>
+        <v>506</v>
       </c>
       <c r="H57" t="s">
-        <v>518</v>
+        <v>509</v>
       </c>
       <c r="I57" t="s">
-        <v>519</v>
+        <v>510</v>
       </c>
       <c r="J57" t="s">
-        <v>515</v>
+        <v>506</v>
       </c>
       <c r="K57" t="s">
-        <v>515</v>
+        <v>506</v>
       </c>
       <c r="L57" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>520</v>
-      </c>
-      <c r="B58" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="58" spans="1:26" ht="203.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B58" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="C58" t="s">
-        <v>521</v>
-      </c>
-      <c r="D58" t="s">
-        <v>522</v>
-      </c>
-      <c r="E58" t="s">
-        <v>523</v>
-      </c>
-      <c r="F58" t="s">
-        <v>524</v>
-      </c>
-      <c r="G58" t="s">
-        <v>525</v>
-      </c>
-      <c r="H58" t="s">
-        <v>526</v>
-      </c>
-      <c r="I58" t="s">
-        <v>527</v>
-      </c>
-      <c r="J58" t="s">
-        <v>521</v>
-      </c>
-      <c r="K58" t="s">
-        <v>528</v>
-      </c>
-      <c r="L58" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C58" s="4" t="s">
+        <v>644</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>645</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>646</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>647</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>648</v>
+      </c>
+      <c r="H58" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="I58" s="4" t="s">
+        <v>650</v>
+      </c>
+      <c r="J58" s="4" t="s">
+        <v>644</v>
+      </c>
+      <c r="K58" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="L58" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="M58" s="6"/>
+      <c r="N58" s="6"/>
+      <c r="O58" s="6"/>
+      <c r="P58" s="6"/>
+      <c r="Q58" s="6"/>
+      <c r="R58" s="6"/>
+      <c r="S58" s="6"/>
+      <c r="T58" s="6"/>
+      <c r="U58" s="6"/>
+      <c r="V58" s="6"/>
+      <c r="W58" s="6"/>
+      <c r="X58" s="6"/>
+      <c r="Y58" s="6"/>
+      <c r="Z58" s="6"/>
+    </row>
+    <row r="59" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>530</v>
+        <v>512</v>
       </c>
       <c r="B59" t="s">
         <v>465</v>
       </c>
       <c r="C59" t="s">
-        <v>531</v>
+        <v>513</v>
       </c>
       <c r="D59" t="s">
-        <v>532</v>
+        <v>514</v>
       </c>
       <c r="E59" t="s">
-        <v>533</v>
+        <v>515</v>
       </c>
       <c r="F59" t="s">
-        <v>534</v>
+        <v>516</v>
       </c>
       <c r="G59" t="s">
-        <v>535</v>
+        <v>517</v>
       </c>
       <c r="H59" t="s">
-        <v>536</v>
+        <v>518</v>
       </c>
       <c r="I59" t="s">
-        <v>537</v>
+        <v>519</v>
       </c>
       <c r="J59" t="s">
-        <v>531</v>
+        <v>513</v>
       </c>
       <c r="K59" t="s">
-        <v>538</v>
+        <v>520</v>
       </c>
       <c r="L59" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="60" spans="1:26" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>540</v>
+        <v>522</v>
       </c>
       <c r="B60" t="s">
         <v>465</v>
       </c>
       <c r="C60" t="s">
-        <v>541</v>
+        <v>523</v>
       </c>
       <c r="D60" t="s">
-        <v>542</v>
+        <v>524</v>
       </c>
       <c r="E60" t="s">
-        <v>543</v>
+        <v>525</v>
       </c>
       <c r="F60" t="s">
-        <v>544</v>
+        <v>526</v>
       </c>
       <c r="G60" t="s">
-        <v>545</v>
+        <v>527</v>
       </c>
       <c r="H60" t="s">
-        <v>546</v>
+        <v>528</v>
       </c>
       <c r="I60" t="s">
-        <v>547</v>
+        <v>529</v>
       </c>
       <c r="J60" t="s">
-        <v>541</v>
+        <v>523</v>
       </c>
       <c r="K60" t="s">
-        <v>548</v>
+        <v>530</v>
       </c>
       <c r="L60" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>550</v>
-      </c>
-      <c r="B61" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="61" spans="1:26" ht="90" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="B61" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="C61" t="s">
-        <v>551</v>
-      </c>
-      <c r="D61" t="s">
-        <v>551</v>
-      </c>
-      <c r="E61" t="s">
-        <v>552</v>
-      </c>
-      <c r="F61" t="s">
-        <v>552</v>
-      </c>
-      <c r="G61" t="s">
-        <v>551</v>
-      </c>
-      <c r="H61" t="s">
-        <v>553</v>
-      </c>
-      <c r="I61" t="s">
-        <v>554</v>
-      </c>
-      <c r="J61" t="s">
-        <v>551</v>
-      </c>
-      <c r="K61" t="s">
-        <v>551</v>
-      </c>
-      <c r="L61" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>555</v>
-      </c>
-      <c r="B62" t="s">
+      <c r="C61" s="4" t="s">
+        <v>662</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>662</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>663</v>
+      </c>
+      <c r="F61" s="3" t="s">
+        <v>663</v>
+      </c>
+      <c r="G61" s="4" t="s">
+        <v>662</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="I61" s="3" t="s">
+        <v>665</v>
+      </c>
+      <c r="J61" s="4" t="s">
+        <v>662</v>
+      </c>
+      <c r="K61" s="4" t="s">
+        <v>662</v>
+      </c>
+      <c r="L61" s="4" t="s">
+        <v>662</v>
+      </c>
+      <c r="M61" s="6"/>
+      <c r="N61" s="6"/>
+      <c r="O61" s="6"/>
+      <c r="P61" s="6"/>
+      <c r="Q61" s="6"/>
+      <c r="R61" s="6"/>
+      <c r="S61" s="6"/>
+      <c r="T61" s="6"/>
+      <c r="U61" s="6"/>
+      <c r="V61" s="6"/>
+      <c r="W61" s="6"/>
+      <c r="X61" s="6"/>
+      <c r="Y61" s="6"/>
+      <c r="Z61" s="6"/>
+    </row>
+    <row r="62" spans="1:26" ht="149.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="B62" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="C62" t="s">
-        <v>556</v>
-      </c>
-      <c r="D62" t="s">
-        <v>557</v>
-      </c>
-      <c r="E62" t="s">
-        <v>558</v>
-      </c>
-      <c r="F62" t="s">
-        <v>559</v>
-      </c>
-      <c r="G62" t="s">
-        <v>560</v>
-      </c>
-      <c r="H62" t="s">
-        <v>561</v>
-      </c>
-      <c r="I62" t="s">
-        <v>562</v>
-      </c>
-      <c r="J62" t="s">
-        <v>556</v>
-      </c>
-      <c r="K62" t="s">
-        <v>563</v>
-      </c>
-      <c r="L62" t="s">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C62" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>655</v>
+      </c>
+      <c r="F62" s="4" t="s">
+        <v>656</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>657</v>
+      </c>
+      <c r="H62" s="4" t="s">
+        <v>658</v>
+      </c>
+      <c r="I62" s="4" t="s">
+        <v>659</v>
+      </c>
+      <c r="J62" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="K62" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="L62" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="M62" s="6"/>
+      <c r="N62" s="6"/>
+      <c r="O62" s="6"/>
+      <c r="P62" s="6"/>
+      <c r="Q62" s="6"/>
+      <c r="R62" s="6"/>
+      <c r="S62" s="6"/>
+      <c r="T62" s="6"/>
+      <c r="U62" s="6"/>
+      <c r="V62" s="6"/>
+      <c r="W62" s="6"/>
+      <c r="X62" s="6"/>
+      <c r="Y62" s="6"/>
+      <c r="Z62" s="6"/>
+    </row>
+    <row r="63" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>565</v>
+        <v>534</v>
       </c>
       <c r="B63" t="s">
         <v>465</v>
       </c>
       <c r="C63" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="D63" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="E63" t="s">
-        <v>567</v>
+        <v>536</v>
       </c>
       <c r="F63" t="s">
-        <v>567</v>
+        <v>536</v>
       </c>
       <c r="G63" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="H63" t="s">
-        <v>568</v>
+        <v>537</v>
       </c>
       <c r="I63" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="J63" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="K63" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="L63" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="64" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>569</v>
+        <v>538</v>
       </c>
       <c r="B64" t="s">
         <v>465</v>
       </c>
       <c r="C64" t="s">
-        <v>570</v>
+        <v>539</v>
       </c>
       <c r="D64" t="s">
-        <v>570</v>
+        <v>539</v>
       </c>
       <c r="E64" t="s">
-        <v>571</v>
+        <v>540</v>
       </c>
       <c r="F64" t="s">
-        <v>572</v>
+        <v>541</v>
       </c>
       <c r="G64" t="s">
-        <v>570</v>
+        <v>539</v>
       </c>
       <c r="H64" t="s">
-        <v>573</v>
+        <v>542</v>
       </c>
       <c r="I64" t="s">
-        <v>574</v>
+        <v>543</v>
       </c>
       <c r="J64" t="s">
-        <v>570</v>
+        <v>539</v>
       </c>
       <c r="K64" t="s">
-        <v>575</v>
+        <v>544</v>
       </c>
       <c r="L64" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="65" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>577</v>
+        <v>546</v>
       </c>
       <c r="B65" t="s">
         <v>465</v>
       </c>
       <c r="C65" t="s">
-        <v>578</v>
+        <v>547</v>
       </c>
       <c r="D65" t="s">
-        <v>579</v>
+        <v>548</v>
       </c>
       <c r="E65" t="s">
-        <v>580</v>
+        <v>549</v>
       </c>
       <c r="F65" t="s">
-        <v>581</v>
+        <v>550</v>
       </c>
       <c r="G65" t="s">
-        <v>582</v>
+        <v>551</v>
       </c>
       <c r="H65" t="s">
-        <v>583</v>
+        <v>552</v>
       </c>
       <c r="I65" t="s">
-        <v>584</v>
+        <v>553</v>
       </c>
       <c r="J65" t="s">
-        <v>578</v>
+        <v>547</v>
       </c>
       <c r="K65" t="s">
-        <v>585</v>
+        <v>554</v>
       </c>
       <c r="L65" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="66" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>587</v>
+        <v>556</v>
       </c>
       <c r="B66" t="s">
         <v>465</v>
       </c>
       <c r="C66" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="D66" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="E66" t="s">
-        <v>567</v>
+        <v>536</v>
       </c>
       <c r="F66" t="s">
-        <v>567</v>
+        <v>536</v>
       </c>
       <c r="G66" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="H66" t="s">
-        <v>568</v>
+        <v>537</v>
       </c>
       <c r="I66" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="J66" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="K66" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="L66" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="67" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>588</v>
+        <v>557</v>
       </c>
       <c r="B67" t="s">
         <v>465</v>
       </c>
       <c r="C67" t="s">
-        <v>570</v>
+        <v>539</v>
       </c>
       <c r="D67" t="s">
-        <v>570</v>
+        <v>539</v>
       </c>
       <c r="E67" t="s">
-        <v>571</v>
+        <v>540</v>
       </c>
       <c r="F67" t="s">
-        <v>572</v>
+        <v>541</v>
       </c>
       <c r="G67" t="s">
-        <v>570</v>
+        <v>539</v>
       </c>
       <c r="H67" t="s">
-        <v>573</v>
+        <v>542</v>
       </c>
       <c r="I67" t="s">
-        <v>574</v>
+        <v>543</v>
       </c>
       <c r="J67" t="s">
-        <v>570</v>
+        <v>539</v>
       </c>
       <c r="K67" t="s">
-        <v>575</v>
+        <v>544</v>
       </c>
       <c r="L67" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="68" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>589</v>
+        <v>558</v>
       </c>
       <c r="B68" t="s">
         <v>465</v>
       </c>
       <c r="C68" t="s">
-        <v>590</v>
+        <v>559</v>
       </c>
       <c r="D68" t="s">
-        <v>591</v>
+        <v>560</v>
       </c>
       <c r="E68" t="s">
-        <v>592</v>
+        <v>561</v>
       </c>
       <c r="F68" t="s">
-        <v>593</v>
+        <v>562</v>
       </c>
       <c r="G68" t="s">
-        <v>594</v>
+        <v>563</v>
       </c>
       <c r="H68" t="s">
-        <v>595</v>
+        <v>564</v>
       </c>
       <c r="I68" t="s">
-        <v>596</v>
+        <v>565</v>
       </c>
       <c r="J68" t="s">
-        <v>590</v>
+        <v>559</v>
       </c>
       <c r="K68" t="s">
-        <v>597</v>
+        <v>566</v>
       </c>
       <c r="L68" t="s">
-        <v>598</v>
-      </c>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="69" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>599</v>
+        <v>568</v>
       </c>
       <c r="B69" t="s">
         <v>465</v>
       </c>
       <c r="C69" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="D69" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="E69" t="s">
-        <v>567</v>
+        <v>536</v>
       </c>
       <c r="F69" t="s">
-        <v>567</v>
+        <v>536</v>
       </c>
       <c r="G69" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="H69" t="s">
-        <v>568</v>
+        <v>537</v>
       </c>
       <c r="I69" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="J69" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="K69" t="s">
-        <v>566</v>
+        <v>535</v>
       </c>
       <c r="L69" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="70" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>600</v>
+        <v>569</v>
       </c>
       <c r="B70" t="s">
         <v>465</v>
       </c>
       <c r="C70" t="s">
+        <v>539</v>
+      </c>
+      <c r="D70" t="s">
+        <v>539</v>
+      </c>
+      <c r="E70" t="s">
+        <v>540</v>
+      </c>
+      <c r="F70" t="s">
+        <v>541</v>
+      </c>
+      <c r="G70" t="s">
+        <v>539</v>
+      </c>
+      <c r="H70" t="s">
+        <v>542</v>
+      </c>
+      <c r="I70" t="s">
+        <v>543</v>
+      </c>
+      <c r="J70" t="s">
+        <v>539</v>
+      </c>
+      <c r="K70" t="s">
+        <v>544</v>
+      </c>
+      <c r="L70" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="71" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>570</v>
-      </c>
-      <c r="D70" t="s">
-        <v>570</v>
-      </c>
-      <c r="E70" t="s">
-        <v>571</v>
-      </c>
-      <c r="F70" t="s">
-        <v>572</v>
-      </c>
-      <c r="G70" t="s">
-        <v>570</v>
-      </c>
-      <c r="H70" t="s">
-        <v>573</v>
-      </c>
-      <c r="I70" t="s">
-        <v>574</v>
-      </c>
-      <c r="J70" t="s">
-        <v>570</v>
-      </c>
-      <c r="K70" t="s">
-        <v>575</v>
-      </c>
-      <c r="L70" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>601</v>
       </c>
       <c r="B71" t="s">
         <v>465</v>
       </c>
       <c r="C71" t="s">
-        <v>602</v>
+        <v>571</v>
       </c>
       <c r="D71" t="s">
-        <v>603</v>
+        <v>572</v>
       </c>
       <c r="E71" t="s">
-        <v>604</v>
+        <v>573</v>
       </c>
       <c r="F71" t="s">
-        <v>605</v>
+        <v>574</v>
       </c>
       <c r="G71" t="s">
-        <v>606</v>
+        <v>575</v>
       </c>
       <c r="H71" t="s">
-        <v>607</v>
+        <v>576</v>
       </c>
       <c r="I71" t="s">
-        <v>608</v>
+        <v>577</v>
       </c>
       <c r="J71" t="s">
-        <v>602</v>
+        <v>571</v>
       </c>
       <c r="K71" t="s">
-        <v>609</v>
+        <v>578</v>
       </c>
       <c r="L71" t="s">
-        <v>610</v>
-      </c>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="72" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>611</v>
+        <v>580</v>
       </c>
       <c r="B72" t="s">
         <v>465</v>
       </c>
       <c r="C72" t="s">
-        <v>612</v>
+        <v>581</v>
       </c>
       <c r="D72" t="s">
-        <v>612</v>
+        <v>581</v>
       </c>
       <c r="E72" t="s">
-        <v>613</v>
+        <v>582</v>
       </c>
       <c r="F72" t="s">
-        <v>614</v>
+        <v>583</v>
       </c>
       <c r="G72" t="s">
-        <v>612</v>
+        <v>581</v>
       </c>
       <c r="H72" t="s">
-        <v>615</v>
+        <v>584</v>
       </c>
       <c r="I72" t="s">
-        <v>616</v>
+        <v>585</v>
       </c>
       <c r="J72" t="s">
-        <v>612</v>
+        <v>581</v>
       </c>
       <c r="K72" t="s">
-        <v>612</v>
+        <v>581</v>
       </c>
       <c r="L72" t="s">
-        <v>612</v>
-      </c>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="73" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>617</v>
+        <v>586</v>
       </c>
       <c r="B73" t="s">
         <v>465</v>
       </c>
       <c r="C73" t="s">
-        <v>618</v>
+        <v>587</v>
       </c>
       <c r="D73" t="s">
-        <v>619</v>
+        <v>588</v>
       </c>
       <c r="E73" t="s">
-        <v>620</v>
+        <v>589</v>
       </c>
       <c r="F73" t="s">
-        <v>621</v>
+        <v>590</v>
       </c>
       <c r="G73" t="s">
-        <v>622</v>
+        <v>591</v>
       </c>
       <c r="H73" t="s">
-        <v>623</v>
+        <v>592</v>
       </c>
       <c r="I73" t="s">
-        <v>624</v>
+        <v>593</v>
       </c>
       <c r="J73" t="s">
-        <v>618</v>
+        <v>587</v>
       </c>
       <c r="K73" t="s">
-        <v>625</v>
+        <v>594</v>
       </c>
       <c r="L73" t="s">
-        <v>626</v>
-      </c>
-    </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="74" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>627</v>
+        <v>596</v>
       </c>
       <c r="B74" t="s">
         <v>465</v>
       </c>
       <c r="C74" t="s">
-        <v>628</v>
+        <v>597</v>
       </c>
       <c r="D74" t="s">
-        <v>628</v>
+        <v>597</v>
       </c>
       <c r="E74" t="s">
-        <v>629</v>
+        <v>598</v>
       </c>
       <c r="F74" t="s">
-        <v>630</v>
+        <v>599</v>
       </c>
       <c r="G74" t="s">
-        <v>628</v>
+        <v>597</v>
       </c>
       <c r="H74" t="s">
-        <v>631</v>
+        <v>600</v>
       </c>
       <c r="I74" t="s">
-        <v>632</v>
+        <v>601</v>
       </c>
       <c r="J74" t="s">
-        <v>628</v>
+        <v>597</v>
       </c>
       <c r="K74" t="s">
-        <v>633</v>
+        <v>602</v>
       </c>
       <c r="L74" t="s">
-        <v>634</v>
-      </c>
-    </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="75" spans="1:26" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>635</v>
+        <v>604</v>
       </c>
       <c r="B75" t="s">
         <v>465</v>
       </c>
       <c r="C75" t="s">
-        <v>636</v>
+        <v>605</v>
       </c>
       <c r="D75" t="s">
-        <v>637</v>
+        <v>606</v>
       </c>
       <c r="E75" t="s">
-        <v>638</v>
+        <v>607</v>
       </c>
       <c r="F75" t="s">
-        <v>639</v>
+        <v>608</v>
       </c>
       <c r="G75" t="s">
-        <v>640</v>
+        <v>609</v>
       </c>
       <c r="H75" t="s">
-        <v>641</v>
+        <v>610</v>
       </c>
       <c r="I75" t="s">
-        <v>642</v>
+        <v>611</v>
       </c>
       <c r="J75" t="s">
-        <v>636</v>
+        <v>605</v>
       </c>
       <c r="K75" t="s">
-        <v>643</v>
+        <v>612</v>
       </c>
       <c r="L75" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="76" spans="1:12" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>645</v>
-      </c>
-      <c r="B76" t="s">
-        <v>646</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>659</v>
-      </c>
-      <c r="D76" s="1" t="s">
-        <v>657</v>
-      </c>
-      <c r="E76" s="1" t="s">
-        <v>660</v>
-      </c>
-      <c r="F76" s="1" t="s">
-        <v>661</v>
-      </c>
-      <c r="G76" s="1" t="s">
-        <v>662</v>
-      </c>
-      <c r="H76" s="1" t="s">
-        <v>663</v>
-      </c>
-      <c r="I76" s="1" t="s">
-        <v>658</v>
-      </c>
-      <c r="J76" s="1" t="s">
-        <v>659</v>
-      </c>
-      <c r="K76" s="1" t="s">
-        <v>664</v>
-      </c>
-      <c r="L76" s="1" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="76" spans="1:26" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="1" t="s">
+        <v>614</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>626</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>627</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>628</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>629</v>
+      </c>
+      <c r="G76" s="3" t="s">
+        <v>630</v>
+      </c>
+      <c r="H76" s="3" t="s">
+        <v>631</v>
+      </c>
+      <c r="I76" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="J76" s="3" t="s">
+        <v>626</v>
+      </c>
+      <c r="K76" s="3" t="s">
+        <v>633</v>
+      </c>
+      <c r="L76" s="5" t="s">
+        <v>634</v>
+      </c>
+      <c r="M76" s="6"/>
+      <c r="N76" s="6"/>
+      <c r="O76" s="6"/>
+      <c r="P76" s="6"/>
+      <c r="Q76" s="6"/>
+      <c r="R76" s="6"/>
+      <c r="S76" s="6"/>
+      <c r="T76" s="6"/>
+      <c r="U76" s="6"/>
+      <c r="V76" s="6"/>
+      <c r="W76" s="6"/>
+      <c r="X76" s="6"/>
+      <c r="Y76" s="6"/>
+      <c r="Z76" s="6"/>
+    </row>
+    <row r="77" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>647</v>
+        <v>616</v>
       </c>
       <c r="B77" t="s">
-        <v>646</v>
+        <v>615</v>
       </c>
       <c r="C77" t="s">
-        <v>648</v>
+        <v>617</v>
       </c>
       <c r="D77" t="s">
-        <v>649</v>
+        <v>618</v>
       </c>
       <c r="E77" t="s">
-        <v>650</v>
+        <v>619</v>
       </c>
       <c r="F77" t="s">
-        <v>651</v>
+        <v>620</v>
       </c>
       <c r="G77" t="s">
-        <v>652</v>
+        <v>621</v>
       </c>
       <c r="H77" t="s">
-        <v>653</v>
+        <v>622</v>
       </c>
       <c r="I77" t="s">
-        <v>654</v>
+        <v>623</v>
       </c>
       <c r="J77" t="s">
-        <v>648</v>
+        <v>617</v>
       </c>
       <c r="K77" t="s">
-        <v>655</v>
+        <v>624</v>
       </c>
       <c r="L77" t="s">
-        <v>656</v>
+        <v>625</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L75 A77:L77 A76" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L55 A77:L77 A57:L57 A59:L60 A63:L75" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>